<commit_message>
added sticker tables and ripples_right
</commit_message>
<xml_diff>
--- a/tables/tables.xlsx
+++ b/tables/tables.xlsx
@@ -5,18 +5,19 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/justindudley/dev/cube/Alg_Slice_And_Widen_daddy/alg-slice-and-widen/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/justindudley/dev/cube/Alg_Slice_And_Widen_daddy/alg-slice-and-widen/tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5487746E-BE80-5142-8848-F1069161C0EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5304ECAB-EBE3-2843-BC41-7EDACA456C5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1400" windowWidth="32260" windowHeight="16800" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1400" windowWidth="32260" windowHeight="16800" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="intermediate" sheetId="2" r:id="rId1"/>
     <sheet name="Other Tables" sheetId="12" r:id="rId2"/>
     <sheet name="basics" sheetId="13" r:id="rId3"/>
-    <sheet name="transformations" sheetId="14" r:id="rId4"/>
+    <sheet name="WCR_Ripples_Left" sheetId="14" r:id="rId4"/>
+    <sheet name="WCR_Ripples_Right" sheetId="15" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -61,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1771" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1784" uniqueCount="268">
   <si>
     <t>The lock password is "password"</t>
   </si>
@@ -838,6 +839,33 @@
   </si>
   <si>
     <t>AZ'--&gt;Z'B</t>
+  </si>
+  <si>
+    <t>XA--&gt;BX</t>
+  </si>
+  <si>
+    <t>X2A--&gt;BX2</t>
+  </si>
+  <si>
+    <t>X'A--&gt;BX'</t>
+  </si>
+  <si>
+    <t>YA--&gt;BY</t>
+  </si>
+  <si>
+    <t>Y2A--&gt;BY2</t>
+  </si>
+  <si>
+    <t>ZA--&gt;BZ</t>
+  </si>
+  <si>
+    <t>Z2A--&gt;BZ2</t>
+  </si>
+  <si>
+    <t>Z'A--&gt;BZ'</t>
+  </si>
+  <si>
+    <t>Y'A--&gt;BY'</t>
   </si>
 </sst>
 </file>
@@ -998,7 +1026,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="65">
+  <dxfs count="79">
     <dxf>
       <fill>
         <patternFill>
@@ -1012,6 +1040,64 @@
           <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1625,25 +1711,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{39DC8717-F9C8-4F69-BEFA-7A9CFBE9E0FC}" name="Table1" displayName="Table1" ref="E4:F58" totalsRowShown="0" headerRowDxfId="64" dataDxfId="63">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{39DC8717-F9C8-4F69-BEFA-7A9CFBE9E0FC}" name="Table1" displayName="Table1" ref="E4:F58" totalsRowShown="0" headerRowDxfId="78" dataDxfId="77">
   <autoFilter ref="E4:F58" xr:uid="{39DC8717-F9C8-4F69-BEFA-7A9CFBE9E0FC}"/>
   <tableColumns count="2">
-    <tableColumn id="2" xr3:uid="{261FAE33-952B-4602-B772-C5B266CD69CD}" name="orig" dataDxfId="62"/>
-    <tableColumn id="3" xr3:uid="{224443CF-22EE-4BA6-97C6-DBE87AE0E5AB}" name="(Y)" dataDxfId="61"/>
+    <tableColumn id="2" xr3:uid="{261FAE33-952B-4602-B772-C5B266CD69CD}" name="orig" dataDxfId="76"/>
+    <tableColumn id="3" xr3:uid="{224443CF-22EE-4BA6-97C6-DBE87AE0E5AB}" name="(Y)" dataDxfId="75"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{45FBC010-C539-3A49-B472-CEB78074ED61}" name="Table17" displayName="Table17" ref="S4:W10" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31" tableBorderDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{45FBC010-C539-3A49-B472-CEB78074ED61}" name="Table17" displayName="Table17" ref="S4:W10" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45" tableBorderDxfId="44">
   <autoFilter ref="S4:W10" xr:uid="{45FBC010-C539-3A49-B472-CEB78074ED61}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{A1DEABE7-CEFF-E149-AE49-24DCA94B2423}" name="Types" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{CFF53E1A-5317-E744-9C39-C222A1DD1142}" name="Groups" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{371F35C8-1153-D447-B1EB-A989F413B950}" name="Thumbs" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{1F12399E-46C3-B241-817A-EF4A9CBCB7ED}" name="U-F centers" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{FE700833-8B7B-BA43-83A9-4E104B315659}" name="180 swaps" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{A1DEABE7-CEFF-E149-AE49-24DCA94B2423}" name="Types" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{CFF53E1A-5317-E744-9C39-C222A1DD1142}" name="Groups" dataDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{371F35C8-1153-D447-B1EB-A989F413B950}" name="Thumbs" dataDxfId="41"/>
+    <tableColumn id="4" xr3:uid="{1F12399E-46C3-B241-817A-EF4A9CBCB7ED}" name="U-F centers" dataDxfId="40"/>
+    <tableColumn id="5" xr3:uid="{FE700833-8B7B-BA43-83A9-4E104B315659}" name="180 swaps" dataDxfId="39"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1657,7 +1743,7 @@
     <tableColumn id="2" xr3:uid="{CD94FC21-7443-0144-9A70-9365970941BA}" name="Y"/>
     <tableColumn id="3" xr3:uid="{171AF67D-A22B-A245-92FB-C5AADC4C7AE7}" name="Z"/>
     <tableColumn id="4" xr3:uid="{AF3D6317-92EA-0E42-8423-B81B14786204}" name="RotationNum"/>
-    <tableColumn id="5" xr3:uid="{AD4E9410-2554-C14B-9833-BFD6234D044D}" name="CompRotationNum" dataDxfId="24">
+    <tableColumn id="5" xr3:uid="{AD4E9410-2554-C14B-9833-BFD6234D044D}" name="CompRotationNum" dataDxfId="38">
       <calculatedColumnFormula>MOD(4-Table14[[#This Row],[RotationNum]],4)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1666,59 +1752,59 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{C5755446-5EF2-8143-8C87-1A7ABBC21F39}" name="Table9" displayName="Table9" ref="A1:D55" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22" tableBorderDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{C5755446-5EF2-8143-8C87-1A7ABBC21F39}" name="Table9" displayName="Table9" ref="A1:D55" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36" tableBorderDxfId="35">
   <autoFilter ref="A1:D55" xr:uid="{C5755446-5EF2-8143-8C87-1A7ABBC21F39}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{6D6CEE8D-9ABA-1D4C-80BC-0111D5EBDB36}" name="orig" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{051D478E-0904-4B06-9033-9E911DE61016}" name="inverse" dataDxfId="19"/>
-    <tableColumn id="11" xr3:uid="{B435DF90-3F4A-0D44-B7C7-981F4EA63919}" name="Complement" dataDxfId="18"/>
-    <tableColumn id="10" xr3:uid="{1C37F64A-F270-DF44-B8D4-BC724CBAFEB0}" name="Rotation Direction" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{6D6CEE8D-9ABA-1D4C-80BC-0111D5EBDB36}" name="orig" dataDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{051D478E-0904-4B06-9033-9E911DE61016}" name="inverse" dataDxfId="33"/>
+    <tableColumn id="11" xr3:uid="{B435DF90-3F4A-0D44-B7C7-981F4EA63919}" name="Complement" dataDxfId="32"/>
+    <tableColumn id="10" xr3:uid="{1C37F64A-F270-DF44-B8D4-BC724CBAFEB0}" name="Rotation Direction" dataDxfId="31"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BD2989BD-C98E-9A41-B671-F66D33543D5A}" name="Table2" displayName="Table2" ref="A1:M55" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BD2989BD-C98E-9A41-B671-F66D33543D5A}" name="Table2" displayName="Table2" ref="A1:M55" totalsRowShown="0" headerRowDxfId="30" dataDxfId="29">
   <autoFilter ref="A1:M55" xr:uid="{BD2989BD-C98E-9A41-B671-F66D33543D5A}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{D84713D4-EBFB-F741-89E9-DF0DE975DCB4}" name="orig" dataDxfId="14">
+    <tableColumn id="1" xr3:uid="{D84713D4-EBFB-F741-89E9-DF0DE975DCB4}" name="orig" dataDxfId="28">
       <calculatedColumnFormula>intermediate!E5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{E90E5CA9-DCC9-A34E-862E-3A065DC3B0EB}" name="AX--&gt;XB" dataDxfId="13">
+    <tableColumn id="7" xr3:uid="{E90E5CA9-DCC9-A34E-862E-3A065DC3B0EB}" name="AX--&gt;XB" dataDxfId="27">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(Table2[[#This Row],[orig]], Table4[orig]), Table4[(X)])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{575DDDB4-7687-FC47-8C90-00126ED99A10}" name="AX2--&gt;X2B" dataDxfId="12">
+    <tableColumn id="6" xr3:uid="{575DDDB4-7687-FC47-8C90-00126ED99A10}" name="AX2--&gt;X2B" dataDxfId="26">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(B2, Table4[orig]), Table4[(X)])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{5EF59DDD-4B53-DE42-B6BD-7FD3D37998AA}" name="AX'--&gt;X'B" dataDxfId="11">
+    <tableColumn id="5" xr3:uid="{5EF59DDD-4B53-DE42-B6BD-7FD3D37998AA}" name="AX'--&gt;X'B" dataDxfId="25">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(C2, Table4[orig]), Table4[(X)])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{2BDA21B0-DDFA-A943-9AE3-2002F487E936}" name="AY--&gt;YB" dataDxfId="10">
+    <tableColumn id="2" xr3:uid="{2BDA21B0-DDFA-A943-9AE3-2002F487E936}" name="AY--&gt;YB" dataDxfId="24">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(A2, Table1[orig]), Table1[(Y)])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{6F2E5D26-C57A-C544-B6C7-D582616ADE53}" name="AY2--&gt;Y2B" dataDxfId="9">
+    <tableColumn id="3" xr3:uid="{6F2E5D26-C57A-C544-B6C7-D582616ADE53}" name="AY2--&gt;Y2B" dataDxfId="23">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(E2, Table1[orig]), Table1[(Y)])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{AF4715C6-E998-8347-9945-E4CECCAC0DF5}" name="AY'--&gt;Y'B" dataDxfId="8">
+    <tableColumn id="4" xr3:uid="{AF4715C6-E998-8347-9945-E4CECCAC0DF5}" name="AY'--&gt;Y'B" dataDxfId="22">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(F2, Table1[orig]), Table1[(Y)])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{B6211330-7C2D-6846-9131-5A50C0C80D28}" name="AZ--&gt;ZB" dataDxfId="7">
+    <tableColumn id="13" xr3:uid="{B6211330-7C2D-6846-9131-5A50C0C80D28}" name="AZ--&gt;ZB" dataDxfId="21">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(Table2[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{5337B581-3138-E343-A346-D938E5793A56}" name="AZ2--&gt;Z2B" dataDxfId="6">
+    <tableColumn id="12" xr3:uid="{5337B581-3138-E343-A346-D938E5793A56}" name="AZ2--&gt;Z2B" dataDxfId="20">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(H2, Table3[orig]), Table3[(Z)])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{7BB96A9A-0D83-DA47-BC99-B547A51EEB37}" name="AZ'--&gt;Z'B" dataDxfId="5">
+    <tableColumn id="11" xr3:uid="{7BB96A9A-0D83-DA47-BC99-B547A51EEB37}" name="AZ'--&gt;Z'B" dataDxfId="19">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(I2, Table3[orig]), Table3[(Z)])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{6E619BEB-3249-F647-8EA6-670CD967F369}" name="T-reflection" dataDxfId="4">
+    <tableColumn id="10" xr3:uid="{6E619BEB-3249-F647-8EA6-670CD967F369}" name="T-reflection" dataDxfId="18">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(Table2[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{345D2781-29F7-BC49-B9CA-B635C564ED1D}" name="H-reflection" dataDxfId="3">
+    <tableColumn id="9" xr3:uid="{345D2781-29F7-BC49-B9CA-B635C564ED1D}" name="H-reflection" dataDxfId="17">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(Table2[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{425EF2DE-6131-C243-9903-CE2FE2C7566D}" name="S-reflection" dataDxfId="2">
+    <tableColumn id="8" xr3:uid="{425EF2DE-6131-C243-9903-CE2FE2C7566D}" name="S-reflection" dataDxfId="16">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(Table2[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1726,63 +1812,109 @@
 </table>
 </file>
 
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA31BBF2-F844-2B4A-9538-D46D7CB98523}" name="Table29" displayName="Table29" ref="A1:M55" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+  <autoFilter ref="A1:M55" xr:uid="{FA31BBF2-F844-2B4A-9538-D46D7CB98523}"/>
+  <tableColumns count="13">
+    <tableColumn id="1" xr3:uid="{EECF3703-E2A6-9F48-BE3F-25177F163AE3}" name="orig" dataDxfId="13">
+      <calculatedColumnFormula>intermediate!E5</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="15" xr3:uid="{261B244F-37C8-E54C-ABB3-FC8E1B40087C}" name="XA--&gt;BX">
+      <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(C2, Table4[orig]), Table4[(X)])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="7" xr3:uid="{9038DD64-8C68-B841-AC8D-A03717F69722}" name="X2A--&gt;BX2" dataDxfId="12">
+      <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(D2, Table4[orig]), Table4[(X)])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{073F3903-CC3B-304C-AB25-5E8BA5D64E4D}" name="X'A--&gt;BX'" dataDxfId="11">
+      <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{DAAFF34B-3D0E-5E40-AD59-08E36F7FDDB9}" name="YA--&gt;BY" dataDxfId="10">
+      <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(F2, Table1[orig]), Table1[(Y)])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{8A781C83-039D-8848-BBD2-B040FF614C9F}" name="Y2A--&gt;BY2" dataDxfId="9">
+      <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(G2, Table1[orig]), Table1[(Y)])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{8F60EA43-EFA3-1C44-8EF2-2ED46CE67CBA}" name="Y'A--&gt;BY'" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{F9F3FA15-50D9-B649-8F07-2FD8E739C1F5}" name="ZA--&gt;BZ" dataDxfId="7">
+      <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(I2, Table3[orig]), Table3[(Z)])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="12" xr3:uid="{5819B1CC-2E75-C34C-8A8C-705876D1E530}" name="Z2A--&gt;BZ2" dataDxfId="6">
+      <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(J2, Table3[orig]), Table3[(Z)])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="11" xr3:uid="{C5CE9D16-6412-464F-ADB8-25539BF69349}" name="Z'A--&gt;BZ'" dataDxfId="5">
+      <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="10" xr3:uid="{8C643816-0FE0-F74A-B773-8C378C181F2A}" name="T-reflection" dataDxfId="4">
+      <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="9" xr3:uid="{431F1C9B-D6E0-964C-980A-00E97B2CA5C8}" name="H-reflection" dataDxfId="3">
+      <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{B4724F81-ABA0-F542-B429-77C7EFF5223E}" name="S-reflection" dataDxfId="2">
+      <calculatedColumnFormula array="1">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{FE45DC8B-6C42-8A4F-A431-A22A6834EB22}" name="Table4" displayName="Table4" ref="B4:C58" totalsRowShown="0" headerRowDxfId="60" dataDxfId="59" tableBorderDxfId="58">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{FE45DC8B-6C42-8A4F-A431-A22A6834EB22}" name="Table4" displayName="Table4" ref="B4:C58" totalsRowShown="0" headerRowDxfId="74" dataDxfId="73" tableBorderDxfId="72">
   <autoFilter ref="B4:C58" xr:uid="{FE45DC8B-6C42-8A4F-A431-A22A6834EB22}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{C6340FD7-0F60-764E-B209-042F7E97B32C}" name="orig" dataDxfId="57"/>
-    <tableColumn id="2" xr3:uid="{320E2130-696E-0041-A459-52DE6F924494}" name="(X)" dataDxfId="56"/>
+    <tableColumn id="1" xr3:uid="{C6340FD7-0F60-764E-B209-042F7E97B32C}" name="orig" dataDxfId="71"/>
+    <tableColumn id="2" xr3:uid="{320E2130-696E-0041-A459-52DE6F924494}" name="(X)" dataDxfId="70"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3B810B22-54A4-6E4E-BF42-E89E63719305}" name="Table3" displayName="Table3" ref="H4:I58" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54" tableBorderDxfId="53">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3B810B22-54A4-6E4E-BF42-E89E63719305}" name="Table3" displayName="Table3" ref="H4:I58" totalsRowShown="0" headerRowDxfId="69" dataDxfId="68" tableBorderDxfId="67">
   <autoFilter ref="H4:I58" xr:uid="{3B810B22-54A4-6E4E-BF42-E89E63719305}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{4640F449-0D6D-6040-93D0-F3F2CB213E57}" name="orig" dataDxfId="52"/>
-    <tableColumn id="2" xr3:uid="{7ED22FEE-42CD-334B-A724-96967247B8AE}" name="(Z)" dataDxfId="51"/>
+    <tableColumn id="1" xr3:uid="{4640F449-0D6D-6040-93D0-F3F2CB213E57}" name="orig" dataDxfId="66"/>
+    <tableColumn id="2" xr3:uid="{7ED22FEE-42CD-334B-A724-96967247B8AE}" name="(Z)" dataDxfId="65"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{6B6F0EB8-6E4C-D946-B118-0E8E7E2AF251}" name="Table5" displayName="Table5" ref="K4:L58" totalsRowShown="0" headerRowDxfId="50" dataDxfId="49" tableBorderDxfId="48">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{6B6F0EB8-6E4C-D946-B118-0E8E7E2AF251}" name="Table5" displayName="Table5" ref="K4:L58" totalsRowShown="0" headerRowDxfId="64" dataDxfId="63" tableBorderDxfId="62">
   <autoFilter ref="K4:L58" xr:uid="{6B6F0EB8-6E4C-D946-B118-0E8E7E2AF251}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{6DFF3402-A2BB-AC45-A076-9A01D15F8D9E}" name="orig" dataDxfId="47"/>
-    <tableColumn id="2" xr3:uid="{FCE8A85E-7009-AB4F-893B-20D1918F78B9}" name="(T-reflection)" dataDxfId="46"/>
+    <tableColumn id="1" xr3:uid="{6DFF3402-A2BB-AC45-A076-9A01D15F8D9E}" name="orig" dataDxfId="61"/>
+    <tableColumn id="2" xr3:uid="{FCE8A85E-7009-AB4F-893B-20D1918F78B9}" name="(T-reflection)" dataDxfId="60"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FD6D42E3-1540-6546-875D-AB4CBA9C4B78}" name="Table6" displayName="Table6" ref="N4:O58" totalsRowShown="0" headerRowDxfId="45" dataDxfId="44" tableBorderDxfId="43">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FD6D42E3-1540-6546-875D-AB4CBA9C4B78}" name="Table6" displayName="Table6" ref="N4:O58" totalsRowShown="0" headerRowDxfId="59" dataDxfId="58" tableBorderDxfId="57">
   <autoFilter ref="N4:O58" xr:uid="{FD6D42E3-1540-6546-875D-AB4CBA9C4B78}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{331E1CFC-0112-E740-BEB9-D98CE358E25B}" name="orig" dataDxfId="42"/>
-    <tableColumn id="2" xr3:uid="{FC0EE1FC-369D-BD4F-9F7C-4A4AF4365B84}" name="(H-reflection)" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{331E1CFC-0112-E740-BEB9-D98CE358E25B}" name="orig" dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{FC0EE1FC-369D-BD4F-9F7C-4A4AF4365B84}" name="(H-reflection)" dataDxfId="55"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{78AC9367-0D38-DE4F-A57E-AB17C0ADDD69}" name="Table7" displayName="Table7" ref="Q4:R58" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39" tableBorderDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{78AC9367-0D38-DE4F-A57E-AB17C0ADDD69}" name="Table7" displayName="Table7" ref="Q4:R58" totalsRowShown="0" headerRowDxfId="54" dataDxfId="53" tableBorderDxfId="52">
   <autoFilter ref="Q4:R58" xr:uid="{78AC9367-0D38-DE4F-A57E-AB17C0ADDD69}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7E4C4427-BE99-1644-AE98-125DA80C16DC}" name="orig" dataDxfId="37"/>
-    <tableColumn id="2" xr3:uid="{AE305346-7FA8-E641-BEE8-F1D2A1D47C85}" name="(S-reflection)" dataDxfId="36"/>
+    <tableColumn id="1" xr3:uid="{7E4C4427-BE99-1644-AE98-125DA80C16DC}" name="orig" dataDxfId="51"/>
+    <tableColumn id="2" xr3:uid="{AE305346-7FA8-E641-BEE8-F1D2A1D47C85}" name="(S-reflection)" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{E5F4FEEC-D297-E84C-B2DE-86C5D909A908}" name="Table11" displayName="Table11" ref="B4:D58" totalsRowShown="0" headerRowDxfId="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{E5F4FEEC-D297-E84C-B2DE-86C5D909A908}" name="Table11" displayName="Table11" ref="B4:D58" totalsRowShown="0" headerRowDxfId="49">
   <autoFilter ref="B4:D58" xr:uid="{E5F4FEEC-D297-E84C-B2DE-86C5D909A908}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D2E4CF96-ECE3-5F48-8B34-4043D6BE457A}" name="Rotation"/>
@@ -1794,7 +1926,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{7135F4C9-1C7D-BC4F-999F-5FD072560DD7}" name="Table12" displayName="Table12" ref="F4:I58" totalsRowShown="0" headerRowDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{7135F4C9-1C7D-BC4F-999F-5FD072560DD7}" name="Table12" displayName="Table12" ref="F4:I58" totalsRowShown="0" headerRowDxfId="48">
   <autoFilter ref="F4:I58" xr:uid="{7135F4C9-1C7D-BC4F-999F-5FD072560DD7}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{D2650480-6F65-5248-A8A1-E74703193DD3}" name="Face Turn Sought"/>
@@ -1811,7 +1943,7 @@
   <autoFilter ref="L4:Q124" xr:uid="{7AA058E9-C5D8-6840-99D0-CDAAF75936DA}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{7EF6168C-4CA7-6B42-9482-2160663272A1}" name="Coro"/>
-    <tableColumn id="2" xr3:uid="{0AAAD174-C6B8-304E-8BC0-36C58B044819}" name="Type" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{0AAAD174-C6B8-304E-8BC0-36C58B044819}" name="Type" dataDxfId="47"/>
     <tableColumn id="3" xr3:uid="{17196624-4AF9-6444-8BFD-B30CFB4A7099}" name="Group"/>
     <tableColumn id="4" xr3:uid="{31C7BA7B-0DB6-D64B-BEC0-F8C4B36F19ED}" name="thumb pivot"/>
     <tableColumn id="5" xr3:uid="{D74D199A-4D17-F949-85EB-043E9DC226B5}" name="U-F center"/>
@@ -4472,7 +4604,7 @@
         <v>18</v>
       </c>
       <c r="G5" t="e" cm="1">
-        <f t="array" ref="G5">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G5" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H5" t="s">
@@ -4536,7 +4668,7 @@
         <v>45</v>
       </c>
       <c r="G6" t="e" cm="1">
-        <f t="array" ref="G6">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G6" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H6" t="s">
@@ -4643,7 +4775,7 @@
         <v>43</v>
       </c>
       <c r="G8" t="e" cm="1">
-        <f t="array" ref="G8">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G8" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H8" t="s">
@@ -4698,7 +4830,7 @@
         <v>21</v>
       </c>
       <c r="G9" t="e" cm="1">
-        <f t="array" ref="G9">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G9" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H9" t="s">
@@ -4817,7 +4949,7 @@
         <v>20</v>
       </c>
       <c r="G11" t="e" cm="1">
-        <f t="array" ref="G11">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G11" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H11" t="s">
@@ -4860,7 +4992,7 @@
         <v>46</v>
       </c>
       <c r="G12" t="e" cm="1">
-        <f t="array" ref="G12">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G12" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H12" t="s">
@@ -4936,7 +5068,7 @@
         <v>48</v>
       </c>
       <c r="G14" t="e" cm="1">
-        <f t="array" ref="G14">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G14" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H14" t="s">
@@ -4976,7 +5108,7 @@
         <v>19</v>
       </c>
       <c r="G15" t="e" cm="1">
-        <f t="array" ref="G15">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G15" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H15" t="s">
@@ -5065,7 +5197,7 @@
         <v>22</v>
       </c>
       <c r="G17" t="e" cm="1">
-        <f t="array" ref="G17">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G17" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H17" t="s">
@@ -5108,7 +5240,7 @@
         <v>70</v>
       </c>
       <c r="G18" t="e" cm="1">
-        <f t="array" ref="G18">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G18" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H18" t="s">
@@ -5178,7 +5310,7 @@
         <v>67</v>
       </c>
       <c r="G20" t="e" cm="1">
-        <f t="array" ref="G20">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G20" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H20" t="s">
@@ -5224,7 +5356,7 @@
         <v>23</v>
       </c>
       <c r="G21" t="e" cm="1">
-        <f t="array" ref="G21">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G21" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H21" t="s">
@@ -5313,7 +5445,7 @@
         <v>44</v>
       </c>
       <c r="G23" t="e" cm="1">
-        <f t="array" ref="G23">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G23" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H23" t="s">
@@ -5446,7 +5578,7 @@
         <v>27</v>
       </c>
       <c r="G27" t="e" cm="1">
-        <f t="array" ref="G27">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G27" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H27" t="s">
@@ -5515,7 +5647,7 @@
         <v>56</v>
       </c>
       <c r="G29" t="e" cm="1">
-        <f t="array" ref="G29">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G29" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H29" t="s">
@@ -5608,7 +5740,7 @@
         <v>65</v>
       </c>
       <c r="G33" t="e" cm="1">
-        <f t="array" ref="G33">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G33" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H33" t="s">
@@ -5677,7 +5809,7 @@
         <v>68</v>
       </c>
       <c r="G35" t="e" cm="1">
-        <f t="array" ref="G35">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G35" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H35" t="s">
@@ -5770,7 +5902,7 @@
         <v>79</v>
       </c>
       <c r="G39" t="e" cm="1">
-        <f t="array" ref="G39">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G39" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H39" t="s">
@@ -5839,7 +5971,7 @@
         <v>55</v>
       </c>
       <c r="G41" t="e" cm="1">
-        <f t="array" ref="G41">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G41" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H41" t="s">
@@ -5932,7 +6064,7 @@
         <v>28</v>
       </c>
       <c r="G45" t="e" cm="1">
-        <f t="array" ref="G45">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G45" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H45" t="s">
@@ -6001,7 +6133,7 @@
         <v>66</v>
       </c>
       <c r="G47" t="e" cm="1">
-        <f t="array" ref="G47">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G47" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H47" t="s">
@@ -6094,7 +6226,7 @@
         <v>57</v>
       </c>
       <c r="G51" t="e" cm="1">
-        <f t="array" ref="G51">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G51" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H51" t="s">
@@ -6163,7 +6295,7 @@
         <v>80</v>
       </c>
       <c r="G53" t="e" cm="1">
-        <f t="array" ref="G53">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G53" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H53" t="s">
@@ -6256,7 +6388,7 @@
         <v>69</v>
       </c>
       <c r="G57" t="e" cm="1">
-        <f t="array" ref="G57">_xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]), #REF!)</f>
+        <f t="array" ref="G57" xml:space="preserve"> _xlfn.XLOOKUP(TRUE, EXACT(Table12[[#This Row],[Face Turn Sought]], Table9[orig]),#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="H57" t="s">
@@ -11403,4 +11535,2974 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{305D7347-9233-464F-8D08-550D21FDDE4C}">
+  <dimension ref="A1:M55"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A2" t="str">
+        <f>intermediate!E5</f>
+        <v>R</v>
+      </c>
+      <c r="B2" t="str" cm="1">
+        <f t="array" ref="B2">_xlfn.XLOOKUP(TRUE, EXACT(C2, Table4[orig]), Table4[(X)])</f>
+        <v>R</v>
+      </c>
+      <c r="C2" t="str" cm="1">
+        <f t="array" ref="C2">_xlfn.XLOOKUP(TRUE, EXACT(D2, Table4[orig]), Table4[(X)])</f>
+        <v>R</v>
+      </c>
+      <c r="D2" t="str" cm="1">
+        <f t="array" ref="D2">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>R</v>
+      </c>
+      <c r="E2" t="str" cm="1">
+        <f t="array" ref="E2">_xlfn.XLOOKUP(TRUE, EXACT(F2, Table1[orig]), Table1[(Y)])</f>
+        <v>B</v>
+      </c>
+      <c r="F2" t="str" cm="1">
+        <f t="array" ref="F2">_xlfn.XLOOKUP(TRUE, EXACT(G2, Table1[orig]), Table1[(Y)])</f>
+        <v>L</v>
+      </c>
+      <c r="G2" t="str" cm="1">
+        <f t="array" ref="G2">_xlfn.XLOOKUP(TRUE, EXACT(Table29[orig], Table1[orig]), Table1[(Y)])</f>
+        <v>F</v>
+      </c>
+      <c r="H2" t="str" cm="1">
+        <f t="array" ref="H2">_xlfn.XLOOKUP(TRUE, EXACT(I2, Table3[orig]), Table3[(Z)])</f>
+        <v>U</v>
+      </c>
+      <c r="I2" t="str" cm="1">
+        <f t="array" ref="I2">_xlfn.XLOOKUP(TRUE, EXACT(J2, Table3[orig]), Table3[(Z)])</f>
+        <v>L</v>
+      </c>
+      <c r="J2" t="str" cm="1">
+        <f t="array" ref="J2">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>D</v>
+      </c>
+      <c r="K2" t="str" cm="1">
+        <f t="array" ref="K2">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>L'</v>
+      </c>
+      <c r="L2" t="str" cm="1">
+        <f t="array" ref="L2">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>R'</v>
+      </c>
+      <c r="M2" t="str" cm="1">
+        <f t="array" ref="M2">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>R'</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A3" t="str">
+        <f>intermediate!E6</f>
+        <v>r</v>
+      </c>
+      <c r="B3" t="str" cm="1">
+        <f t="array" ref="B3">_xlfn.XLOOKUP(TRUE, EXACT(C3, Table4[orig]), Table4[(X)])</f>
+        <v>r</v>
+      </c>
+      <c r="C3" t="str" cm="1">
+        <f t="array" ref="C3">_xlfn.XLOOKUP(TRUE, EXACT(D3, Table4[orig]), Table4[(X)])</f>
+        <v>r</v>
+      </c>
+      <c r="D3" t="str" cm="1">
+        <f t="array" ref="D3">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>r</v>
+      </c>
+      <c r="E3" t="str" cm="1">
+        <f t="array" ref="E3">_xlfn.XLOOKUP(TRUE, EXACT(F3, Table1[orig]), Table1[(Y)])</f>
+        <v>b</v>
+      </c>
+      <c r="F3" t="str" cm="1">
+        <f t="array" ref="F3">_xlfn.XLOOKUP(TRUE, EXACT(G3, Table1[orig]), Table1[(Y)])</f>
+        <v>l</v>
+      </c>
+      <c r="G3" t="str" cm="1">
+        <f t="array" ref="G3">_xlfn.XLOOKUP(TRUE, EXACT(A3, Table1[orig]), Table1[(Y)])</f>
+        <v>f</v>
+      </c>
+      <c r="H3" t="str" cm="1">
+        <f t="array" ref="H3">_xlfn.XLOOKUP(TRUE, EXACT(I3, Table3[orig]), Table3[(Z)])</f>
+        <v>u</v>
+      </c>
+      <c r="I3" t="str" cm="1">
+        <f t="array" ref="I3">_xlfn.XLOOKUP(TRUE, EXACT(J3, Table3[orig]), Table3[(Z)])</f>
+        <v>l</v>
+      </c>
+      <c r="J3" t="str" cm="1">
+        <f t="array" ref="J3">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>d</v>
+      </c>
+      <c r="K3" t="str" cm="1">
+        <f t="array" ref="K3">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>l'</v>
+      </c>
+      <c r="L3" t="str" cm="1">
+        <f t="array" ref="L3">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>r'</v>
+      </c>
+      <c r="M3" t="str" cm="1">
+        <f t="array" ref="M3">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>r'</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A4" t="str">
+        <f>intermediate!E7</f>
+        <v>T</v>
+      </c>
+      <c r="B4" t="str" cm="1">
+        <f t="array" ref="B4">_xlfn.XLOOKUP(TRUE, EXACT(C4, Table4[orig]), Table4[(X)])</f>
+        <v>T</v>
+      </c>
+      <c r="C4" t="str" cm="1">
+        <f t="array" ref="C4">_xlfn.XLOOKUP(TRUE, EXACT(D4, Table4[orig]), Table4[(X)])</f>
+        <v>T</v>
+      </c>
+      <c r="D4" t="str" cm="1">
+        <f t="array" ref="D4">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>T</v>
+      </c>
+      <c r="E4" t="str" cm="1">
+        <f t="array" ref="E4">_xlfn.XLOOKUP(TRUE, EXACT(F4, Table1[orig]), Table1[(Y)])</f>
+        <v>S'</v>
+      </c>
+      <c r="F4" t="str" cm="1">
+        <f t="array" ref="F4">_xlfn.XLOOKUP(TRUE, EXACT(G4, Table1[orig]), Table1[(Y)])</f>
+        <v>T'</v>
+      </c>
+      <c r="G4" t="str" cm="1">
+        <f t="array" ref="G4">_xlfn.XLOOKUP(TRUE, EXACT(A4, Table1[orig]), Table1[(Y)])</f>
+        <v>S</v>
+      </c>
+      <c r="H4" t="str" cm="1">
+        <f t="array" ref="H4">_xlfn.XLOOKUP(TRUE, EXACT(I4, Table3[orig]), Table3[(Z)])</f>
+        <v>H</v>
+      </c>
+      <c r="I4" t="str" cm="1">
+        <f t="array" ref="I4">_xlfn.XLOOKUP(TRUE, EXACT(J4, Table3[orig]), Table3[(Z)])</f>
+        <v>T'</v>
+      </c>
+      <c r="J4" t="str" cm="1">
+        <f t="array" ref="J4">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>H'</v>
+      </c>
+      <c r="K4" t="str" cm="1">
+        <f t="array" ref="K4">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>T</v>
+      </c>
+      <c r="L4" t="str" cm="1">
+        <f t="array" ref="L4">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>T'</v>
+      </c>
+      <c r="M4" t="str" cm="1">
+        <f t="array" ref="M4">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>T'</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A5" t="str">
+        <f>intermediate!E8</f>
+        <v>l</v>
+      </c>
+      <c r="B5" t="str" cm="1">
+        <f t="array" ref="B5">_xlfn.XLOOKUP(TRUE, EXACT(C5, Table4[orig]), Table4[(X)])</f>
+        <v>l</v>
+      </c>
+      <c r="C5" t="str" cm="1">
+        <f t="array" ref="C5">_xlfn.XLOOKUP(TRUE, EXACT(D5, Table4[orig]), Table4[(X)])</f>
+        <v>l</v>
+      </c>
+      <c r="D5" t="str" cm="1">
+        <f t="array" ref="D5">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>l</v>
+      </c>
+      <c r="E5" t="str" cm="1">
+        <f t="array" ref="E5">_xlfn.XLOOKUP(TRUE, EXACT(F5, Table1[orig]), Table1[(Y)])</f>
+        <v>f</v>
+      </c>
+      <c r="F5" t="str" cm="1">
+        <f t="array" ref="F5">_xlfn.XLOOKUP(TRUE, EXACT(G5, Table1[orig]), Table1[(Y)])</f>
+        <v>r</v>
+      </c>
+      <c r="G5" t="str" cm="1">
+        <f t="array" ref="G5">_xlfn.XLOOKUP(TRUE, EXACT(A5, Table1[orig]), Table1[(Y)])</f>
+        <v>b</v>
+      </c>
+      <c r="H5" t="str" cm="1">
+        <f t="array" ref="H5">_xlfn.XLOOKUP(TRUE, EXACT(I5, Table3[orig]), Table3[(Z)])</f>
+        <v>d</v>
+      </c>
+      <c r="I5" t="str" cm="1">
+        <f t="array" ref="I5">_xlfn.XLOOKUP(TRUE, EXACT(J5, Table3[orig]), Table3[(Z)])</f>
+        <v>r</v>
+      </c>
+      <c r="J5" t="str" cm="1">
+        <f t="array" ref="J5">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>u</v>
+      </c>
+      <c r="K5" t="str" cm="1">
+        <f t="array" ref="K5">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>r'</v>
+      </c>
+      <c r="L5" t="str" cm="1">
+        <f t="array" ref="L5">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>l'</v>
+      </c>
+      <c r="M5" t="str" cm="1">
+        <f t="array" ref="M5">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>l'</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A6" t="str">
+        <f>intermediate!E9</f>
+        <v>L</v>
+      </c>
+      <c r="B6" t="str" cm="1">
+        <f t="array" ref="B6">_xlfn.XLOOKUP(TRUE, EXACT(C6, Table4[orig]), Table4[(X)])</f>
+        <v>L</v>
+      </c>
+      <c r="C6" t="str" cm="1">
+        <f t="array" ref="C6">_xlfn.XLOOKUP(TRUE, EXACT(D6, Table4[orig]), Table4[(X)])</f>
+        <v>L</v>
+      </c>
+      <c r="D6" t="str" cm="1">
+        <f t="array" ref="D6">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>L</v>
+      </c>
+      <c r="E6" t="str" cm="1">
+        <f t="array" ref="E6">_xlfn.XLOOKUP(TRUE, EXACT(F6, Table1[orig]), Table1[(Y)])</f>
+        <v>F</v>
+      </c>
+      <c r="F6" t="str" cm="1">
+        <f t="array" ref="F6">_xlfn.XLOOKUP(TRUE, EXACT(G6, Table1[orig]), Table1[(Y)])</f>
+        <v>R</v>
+      </c>
+      <c r="G6" t="str" cm="1">
+        <f t="array" ref="G6">_xlfn.XLOOKUP(TRUE, EXACT(A6, Table1[orig]), Table1[(Y)])</f>
+        <v>B</v>
+      </c>
+      <c r="H6" t="str" cm="1">
+        <f t="array" ref="H6">_xlfn.XLOOKUP(TRUE, EXACT(I6, Table3[orig]), Table3[(Z)])</f>
+        <v>D</v>
+      </c>
+      <c r="I6" t="str" cm="1">
+        <f t="array" ref="I6">_xlfn.XLOOKUP(TRUE, EXACT(J6, Table3[orig]), Table3[(Z)])</f>
+        <v>R</v>
+      </c>
+      <c r="J6" t="str" cm="1">
+        <f t="array" ref="J6">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>U</v>
+      </c>
+      <c r="K6" t="str" cm="1">
+        <f t="array" ref="K6">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>R'</v>
+      </c>
+      <c r="L6" t="str" cm="1">
+        <f t="array" ref="L6">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>L'</v>
+      </c>
+      <c r="M6" t="str" cm="1">
+        <f t="array" ref="M6">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>L'</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="str">
+        <f>intermediate!E10</f>
+        <v>X</v>
+      </c>
+      <c r="B7" s="3" t="str" cm="1">
+        <f t="array" ref="B7">_xlfn.XLOOKUP(TRUE, EXACT(C7, Table4[orig]), Table4[(X)])</f>
+        <v>X</v>
+      </c>
+      <c r="C7" s="3" t="str" cm="1">
+        <f t="array" ref="C7">_xlfn.XLOOKUP(TRUE, EXACT(D7, Table4[orig]), Table4[(X)])</f>
+        <v>X</v>
+      </c>
+      <c r="D7" s="3" t="str" cm="1">
+        <f t="array" ref="D7">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>X</v>
+      </c>
+      <c r="E7" s="3" t="str" cm="1">
+        <f t="array" ref="E7">_xlfn.XLOOKUP(TRUE, EXACT(F7, Table1[orig]), Table1[(Y)])</f>
+        <v>Z'</v>
+      </c>
+      <c r="F7" s="3" t="str" cm="1">
+        <f t="array" ref="F7">_xlfn.XLOOKUP(TRUE, EXACT(G7, Table1[orig]), Table1[(Y)])</f>
+        <v>X'</v>
+      </c>
+      <c r="G7" s="3" t="str" cm="1">
+        <f t="array" ref="G7">_xlfn.XLOOKUP(TRUE, EXACT(A7, Table1[orig]), Table1[(Y)])</f>
+        <v>Z</v>
+      </c>
+      <c r="H7" s="3" t="str" cm="1">
+        <f t="array" ref="H7">_xlfn.XLOOKUP(TRUE, EXACT(I7, Table3[orig]), Table3[(Z)])</f>
+        <v>Y</v>
+      </c>
+      <c r="I7" s="3" t="str" cm="1">
+        <f t="array" ref="I7">_xlfn.XLOOKUP(TRUE, EXACT(J7, Table3[orig]), Table3[(Z)])</f>
+        <v>X'</v>
+      </c>
+      <c r="J7" s="3" t="str" cm="1">
+        <f t="array" ref="J7">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>Y'</v>
+      </c>
+      <c r="K7" s="3" t="str" cm="1">
+        <f t="array" ref="K7">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>X</v>
+      </c>
+      <c r="L7" s="3" t="str" cm="1">
+        <f t="array" ref="L7">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>X'</v>
+      </c>
+      <c r="M7" s="3" t="str" cm="1">
+        <f t="array" ref="M7">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>X'</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A8" t="str">
+        <f>intermediate!E11</f>
+        <v>R'</v>
+      </c>
+      <c r="B8" t="str" cm="1">
+        <f t="array" ref="B8">_xlfn.XLOOKUP(TRUE, EXACT(C8, Table4[orig]), Table4[(X)])</f>
+        <v>R'</v>
+      </c>
+      <c r="C8" t="str" cm="1">
+        <f t="array" ref="C8">_xlfn.XLOOKUP(TRUE, EXACT(D8, Table4[orig]), Table4[(X)])</f>
+        <v>R'</v>
+      </c>
+      <c r="D8" t="str" cm="1">
+        <f t="array" ref="D8">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>R'</v>
+      </c>
+      <c r="E8" t="str" cm="1">
+        <f t="array" ref="E8">_xlfn.XLOOKUP(TRUE, EXACT(F8, Table1[orig]), Table1[(Y)])</f>
+        <v>B'</v>
+      </c>
+      <c r="F8" t="str" cm="1">
+        <f t="array" ref="F8">_xlfn.XLOOKUP(TRUE, EXACT(G8, Table1[orig]), Table1[(Y)])</f>
+        <v>L'</v>
+      </c>
+      <c r="G8" t="str" cm="1">
+        <f t="array" ref="G8">_xlfn.XLOOKUP(TRUE, EXACT(A8, Table1[orig]), Table1[(Y)])</f>
+        <v>F'</v>
+      </c>
+      <c r="H8" t="str" cm="1">
+        <f t="array" ref="H8">_xlfn.XLOOKUP(TRUE, EXACT(I8, Table3[orig]), Table3[(Z)])</f>
+        <v>U'</v>
+      </c>
+      <c r="I8" t="str" cm="1">
+        <f t="array" ref="I8">_xlfn.XLOOKUP(TRUE, EXACT(J8, Table3[orig]), Table3[(Z)])</f>
+        <v>L'</v>
+      </c>
+      <c r="J8" t="str" cm="1">
+        <f t="array" ref="J8">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>D'</v>
+      </c>
+      <c r="K8" t="str" cm="1">
+        <f t="array" ref="K8">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>L</v>
+      </c>
+      <c r="L8" t="str" cm="1">
+        <f t="array" ref="L8">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>R</v>
+      </c>
+      <c r="M8" t="str" cm="1">
+        <f t="array" ref="M8">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>R</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A9" t="str">
+        <f>intermediate!E12</f>
+        <v>r'</v>
+      </c>
+      <c r="B9" t="str" cm="1">
+        <f t="array" ref="B9">_xlfn.XLOOKUP(TRUE, EXACT(C9, Table4[orig]), Table4[(X)])</f>
+        <v>r'</v>
+      </c>
+      <c r="C9" t="str" cm="1">
+        <f t="array" ref="C9">_xlfn.XLOOKUP(TRUE, EXACT(D9, Table4[orig]), Table4[(X)])</f>
+        <v>r'</v>
+      </c>
+      <c r="D9" t="str" cm="1">
+        <f t="array" ref="D9">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>r'</v>
+      </c>
+      <c r="E9" t="str" cm="1">
+        <f t="array" ref="E9">_xlfn.XLOOKUP(TRUE, EXACT(F9, Table1[orig]), Table1[(Y)])</f>
+        <v>b'</v>
+      </c>
+      <c r="F9" t="str" cm="1">
+        <f t="array" ref="F9">_xlfn.XLOOKUP(TRUE, EXACT(G9, Table1[orig]), Table1[(Y)])</f>
+        <v>l'</v>
+      </c>
+      <c r="G9" t="str" cm="1">
+        <f t="array" ref="G9">_xlfn.XLOOKUP(TRUE, EXACT(A9, Table1[orig]), Table1[(Y)])</f>
+        <v>f'</v>
+      </c>
+      <c r="H9" t="str" cm="1">
+        <f t="array" ref="H9">_xlfn.XLOOKUP(TRUE, EXACT(I9, Table3[orig]), Table3[(Z)])</f>
+        <v>u'</v>
+      </c>
+      <c r="I9" t="str" cm="1">
+        <f t="array" ref="I9">_xlfn.XLOOKUP(TRUE, EXACT(J9, Table3[orig]), Table3[(Z)])</f>
+        <v>l'</v>
+      </c>
+      <c r="J9" t="str" cm="1">
+        <f t="array" ref="J9">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>d'</v>
+      </c>
+      <c r="K9" t="str" cm="1">
+        <f t="array" ref="K9">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>l</v>
+      </c>
+      <c r="L9" t="str" cm="1">
+        <f t="array" ref="L9">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>r</v>
+      </c>
+      <c r="M9" t="str" cm="1">
+        <f t="array" ref="M9">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>r</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A10" t="str">
+        <f>intermediate!E13</f>
+        <v>T'</v>
+      </c>
+      <c r="B10" t="str" cm="1">
+        <f t="array" ref="B10">_xlfn.XLOOKUP(TRUE, EXACT(C10, Table4[orig]), Table4[(X)])</f>
+        <v>T'</v>
+      </c>
+      <c r="C10" t="str" cm="1">
+        <f t="array" ref="C10">_xlfn.XLOOKUP(TRUE, EXACT(D10, Table4[orig]), Table4[(X)])</f>
+        <v>T'</v>
+      </c>
+      <c r="D10" t="str" cm="1">
+        <f t="array" ref="D10">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>T'</v>
+      </c>
+      <c r="E10" t="str" cm="1">
+        <f t="array" ref="E10">_xlfn.XLOOKUP(TRUE, EXACT(F10, Table1[orig]), Table1[(Y)])</f>
+        <v>S</v>
+      </c>
+      <c r="F10" t="str" cm="1">
+        <f t="array" ref="F10">_xlfn.XLOOKUP(TRUE, EXACT(G10, Table1[orig]), Table1[(Y)])</f>
+        <v>T</v>
+      </c>
+      <c r="G10" t="str" cm="1">
+        <f t="array" ref="G10">_xlfn.XLOOKUP(TRUE, EXACT(A10, Table1[orig]), Table1[(Y)])</f>
+        <v>S'</v>
+      </c>
+      <c r="H10" t="str" cm="1">
+        <f t="array" ref="H10">_xlfn.XLOOKUP(TRUE, EXACT(I10, Table3[orig]), Table3[(Z)])</f>
+        <v>H'</v>
+      </c>
+      <c r="I10" t="str" cm="1">
+        <f t="array" ref="I10">_xlfn.XLOOKUP(TRUE, EXACT(J10, Table3[orig]), Table3[(Z)])</f>
+        <v>T</v>
+      </c>
+      <c r="J10" t="str" cm="1">
+        <f t="array" ref="J10">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>H</v>
+      </c>
+      <c r="K10" t="str" cm="1">
+        <f t="array" ref="K10">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>T'</v>
+      </c>
+      <c r="L10" t="str" cm="1">
+        <f t="array" ref="L10">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>T</v>
+      </c>
+      <c r="M10" t="str" cm="1">
+        <f t="array" ref="M10">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>T</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A11" t="str">
+        <f>intermediate!E14</f>
+        <v>l'</v>
+      </c>
+      <c r="B11" t="str" cm="1">
+        <f t="array" ref="B11">_xlfn.XLOOKUP(TRUE, EXACT(C11, Table4[orig]), Table4[(X)])</f>
+        <v>l'</v>
+      </c>
+      <c r="C11" t="str" cm="1">
+        <f t="array" ref="C11">_xlfn.XLOOKUP(TRUE, EXACT(D11, Table4[orig]), Table4[(X)])</f>
+        <v>l'</v>
+      </c>
+      <c r="D11" t="str" cm="1">
+        <f t="array" ref="D11">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>l'</v>
+      </c>
+      <c r="E11" t="str" cm="1">
+        <f t="array" ref="E11">_xlfn.XLOOKUP(TRUE, EXACT(F11, Table1[orig]), Table1[(Y)])</f>
+        <v>f'</v>
+      </c>
+      <c r="F11" t="str" cm="1">
+        <f t="array" ref="F11">_xlfn.XLOOKUP(TRUE, EXACT(G11, Table1[orig]), Table1[(Y)])</f>
+        <v>r'</v>
+      </c>
+      <c r="G11" t="str" cm="1">
+        <f t="array" ref="G11">_xlfn.XLOOKUP(TRUE, EXACT(A11, Table1[orig]), Table1[(Y)])</f>
+        <v>b'</v>
+      </c>
+      <c r="H11" t="str" cm="1">
+        <f t="array" ref="H11">_xlfn.XLOOKUP(TRUE, EXACT(I11, Table3[orig]), Table3[(Z)])</f>
+        <v>d'</v>
+      </c>
+      <c r="I11" t="str" cm="1">
+        <f t="array" ref="I11">_xlfn.XLOOKUP(TRUE, EXACT(J11, Table3[orig]), Table3[(Z)])</f>
+        <v>r'</v>
+      </c>
+      <c r="J11" t="str" cm="1">
+        <f t="array" ref="J11">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>u'</v>
+      </c>
+      <c r="K11" t="str" cm="1">
+        <f t="array" ref="K11">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>r</v>
+      </c>
+      <c r="L11" t="str" cm="1">
+        <f t="array" ref="L11">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>l</v>
+      </c>
+      <c r="M11" t="str" cm="1">
+        <f t="array" ref="M11">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>l</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A12" t="str">
+        <f>intermediate!E15</f>
+        <v>L'</v>
+      </c>
+      <c r="B12" t="str" cm="1">
+        <f t="array" ref="B12">_xlfn.XLOOKUP(TRUE, EXACT(C12, Table4[orig]), Table4[(X)])</f>
+        <v>L'</v>
+      </c>
+      <c r="C12" t="str" cm="1">
+        <f t="array" ref="C12">_xlfn.XLOOKUP(TRUE, EXACT(D12, Table4[orig]), Table4[(X)])</f>
+        <v>L'</v>
+      </c>
+      <c r="D12" t="str" cm="1">
+        <f t="array" ref="D12">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>L'</v>
+      </c>
+      <c r="E12" t="str" cm="1">
+        <f t="array" ref="E12">_xlfn.XLOOKUP(TRUE, EXACT(F12, Table1[orig]), Table1[(Y)])</f>
+        <v>F'</v>
+      </c>
+      <c r="F12" t="str" cm="1">
+        <f t="array" ref="F12">_xlfn.XLOOKUP(TRUE, EXACT(G12, Table1[orig]), Table1[(Y)])</f>
+        <v>R'</v>
+      </c>
+      <c r="G12" t="str" cm="1">
+        <f t="array" ref="G12">_xlfn.XLOOKUP(TRUE, EXACT(A12, Table1[orig]), Table1[(Y)])</f>
+        <v>B'</v>
+      </c>
+      <c r="H12" t="str" cm="1">
+        <f t="array" ref="H12">_xlfn.XLOOKUP(TRUE, EXACT(I12, Table3[orig]), Table3[(Z)])</f>
+        <v>D'</v>
+      </c>
+      <c r="I12" t="str" cm="1">
+        <f t="array" ref="I12">_xlfn.XLOOKUP(TRUE, EXACT(J12, Table3[orig]), Table3[(Z)])</f>
+        <v>R'</v>
+      </c>
+      <c r="J12" t="str" cm="1">
+        <f t="array" ref="J12">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>U'</v>
+      </c>
+      <c r="K12" t="str" cm="1">
+        <f t="array" ref="K12">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>R</v>
+      </c>
+      <c r="L12" t="str" cm="1">
+        <f t="array" ref="L12">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>L</v>
+      </c>
+      <c r="M12" t="str" cm="1">
+        <f t="array" ref="M12">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>L</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="str">
+        <f>intermediate!E16</f>
+        <v>X'</v>
+      </c>
+      <c r="B13" s="3" t="str" cm="1">
+        <f t="array" ref="B13">_xlfn.XLOOKUP(TRUE, EXACT(C13, Table4[orig]), Table4[(X)])</f>
+        <v>X'</v>
+      </c>
+      <c r="C13" s="3" t="str" cm="1">
+        <f t="array" ref="C13">_xlfn.XLOOKUP(TRUE, EXACT(D13, Table4[orig]), Table4[(X)])</f>
+        <v>X'</v>
+      </c>
+      <c r="D13" s="3" t="str" cm="1">
+        <f t="array" ref="D13">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>X'</v>
+      </c>
+      <c r="E13" s="3" t="str" cm="1">
+        <f t="array" ref="E13">_xlfn.XLOOKUP(TRUE, EXACT(F13, Table1[orig]), Table1[(Y)])</f>
+        <v>Z</v>
+      </c>
+      <c r="F13" s="3" t="str" cm="1">
+        <f t="array" ref="F13">_xlfn.XLOOKUP(TRUE, EXACT(G13, Table1[orig]), Table1[(Y)])</f>
+        <v>X</v>
+      </c>
+      <c r="G13" s="3" t="str" cm="1">
+        <f t="array" ref="G13">_xlfn.XLOOKUP(TRUE, EXACT(A13, Table1[orig]), Table1[(Y)])</f>
+        <v>Z'</v>
+      </c>
+      <c r="H13" s="3" t="str" cm="1">
+        <f t="array" ref="H13">_xlfn.XLOOKUP(TRUE, EXACT(I13, Table3[orig]), Table3[(Z)])</f>
+        <v>Y'</v>
+      </c>
+      <c r="I13" s="3" t="str" cm="1">
+        <f t="array" ref="I13">_xlfn.XLOOKUP(TRUE, EXACT(J13, Table3[orig]), Table3[(Z)])</f>
+        <v>X</v>
+      </c>
+      <c r="J13" s="3" t="str" cm="1">
+        <f t="array" ref="J13">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>Y</v>
+      </c>
+      <c r="K13" s="3" t="str" cm="1">
+        <f t="array" ref="K13">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>X'</v>
+      </c>
+      <c r="L13" s="3" t="str" cm="1">
+        <f t="array" ref="L13">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>X</v>
+      </c>
+      <c r="M13" s="3" t="str" cm="1">
+        <f t="array" ref="M13">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>X</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A14" t="str">
+        <f>intermediate!E17</f>
+        <v>R2</v>
+      </c>
+      <c r="B14" t="str" cm="1">
+        <f t="array" ref="B14">_xlfn.XLOOKUP(TRUE, EXACT(C14, Table4[orig]), Table4[(X)])</f>
+        <v>R2</v>
+      </c>
+      <c r="C14" t="str" cm="1">
+        <f t="array" ref="C14">_xlfn.XLOOKUP(TRUE, EXACT(D14, Table4[orig]), Table4[(X)])</f>
+        <v>R2</v>
+      </c>
+      <c r="D14" t="str" cm="1">
+        <f t="array" ref="D14">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>R2</v>
+      </c>
+      <c r="E14" t="str" cm="1">
+        <f t="array" ref="E14">_xlfn.XLOOKUP(TRUE, EXACT(F14, Table1[orig]), Table1[(Y)])</f>
+        <v>B2</v>
+      </c>
+      <c r="F14" t="str" cm="1">
+        <f t="array" ref="F14">_xlfn.XLOOKUP(TRUE, EXACT(G14, Table1[orig]), Table1[(Y)])</f>
+        <v>L2</v>
+      </c>
+      <c r="G14" t="str" cm="1">
+        <f t="array" ref="G14">_xlfn.XLOOKUP(TRUE, EXACT(A14, Table1[orig]), Table1[(Y)])</f>
+        <v>F2</v>
+      </c>
+      <c r="H14" t="str" cm="1">
+        <f t="array" ref="H14">_xlfn.XLOOKUP(TRUE, EXACT(I14, Table3[orig]), Table3[(Z)])</f>
+        <v>U2</v>
+      </c>
+      <c r="I14" t="str" cm="1">
+        <f t="array" ref="I14">_xlfn.XLOOKUP(TRUE, EXACT(J14, Table3[orig]), Table3[(Z)])</f>
+        <v>L2</v>
+      </c>
+      <c r="J14" t="str" cm="1">
+        <f t="array" ref="J14">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>D2</v>
+      </c>
+      <c r="K14" t="str" cm="1">
+        <f t="array" ref="K14">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>L2</v>
+      </c>
+      <c r="L14" t="str" cm="1">
+        <f t="array" ref="L14">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>R2</v>
+      </c>
+      <c r="M14" t="str" cm="1">
+        <f t="array" ref="M14">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>R2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A15" t="str">
+        <f>intermediate!E18</f>
+        <v>r2</v>
+      </c>
+      <c r="B15" t="str" cm="1">
+        <f t="array" ref="B15">_xlfn.XLOOKUP(TRUE, EXACT(C15, Table4[orig]), Table4[(X)])</f>
+        <v>r2</v>
+      </c>
+      <c r="C15" t="str" cm="1">
+        <f t="array" ref="C15">_xlfn.XLOOKUP(TRUE, EXACT(D15, Table4[orig]), Table4[(X)])</f>
+        <v>r2</v>
+      </c>
+      <c r="D15" t="str" cm="1">
+        <f t="array" ref="D15">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>r2</v>
+      </c>
+      <c r="E15" t="str" cm="1">
+        <f t="array" ref="E15">_xlfn.XLOOKUP(TRUE, EXACT(F15, Table1[orig]), Table1[(Y)])</f>
+        <v>b2</v>
+      </c>
+      <c r="F15" t="str" cm="1">
+        <f t="array" ref="F15">_xlfn.XLOOKUP(TRUE, EXACT(G15, Table1[orig]), Table1[(Y)])</f>
+        <v>l2</v>
+      </c>
+      <c r="G15" t="str" cm="1">
+        <f t="array" ref="G15">_xlfn.XLOOKUP(TRUE, EXACT(A15, Table1[orig]), Table1[(Y)])</f>
+        <v>f2</v>
+      </c>
+      <c r="H15" t="str" cm="1">
+        <f t="array" ref="H15">_xlfn.XLOOKUP(TRUE, EXACT(I15, Table3[orig]), Table3[(Z)])</f>
+        <v>u2</v>
+      </c>
+      <c r="I15" t="str" cm="1">
+        <f t="array" ref="I15">_xlfn.XLOOKUP(TRUE, EXACT(J15, Table3[orig]), Table3[(Z)])</f>
+        <v>l2</v>
+      </c>
+      <c r="J15" t="str" cm="1">
+        <f t="array" ref="J15">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>d2</v>
+      </c>
+      <c r="K15" t="str" cm="1">
+        <f t="array" ref="K15">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>l2</v>
+      </c>
+      <c r="L15" t="str" cm="1">
+        <f t="array" ref="L15">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>r2</v>
+      </c>
+      <c r="M15" t="str" cm="1">
+        <f t="array" ref="M15">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>r2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A16" t="str">
+        <f>intermediate!E19</f>
+        <v>T2</v>
+      </c>
+      <c r="B16" t="str" cm="1">
+        <f t="array" ref="B16">_xlfn.XLOOKUP(TRUE, EXACT(C16, Table4[orig]), Table4[(X)])</f>
+        <v>T2</v>
+      </c>
+      <c r="C16" t="str" cm="1">
+        <f t="array" ref="C16">_xlfn.XLOOKUP(TRUE, EXACT(D16, Table4[orig]), Table4[(X)])</f>
+        <v>T2</v>
+      </c>
+      <c r="D16" t="str" cm="1">
+        <f t="array" ref="D16">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>T2</v>
+      </c>
+      <c r="E16" t="str" cm="1">
+        <f t="array" ref="E16">_xlfn.XLOOKUP(TRUE, EXACT(F16, Table1[orig]), Table1[(Y)])</f>
+        <v>S2</v>
+      </c>
+      <c r="F16" t="str" cm="1">
+        <f t="array" ref="F16">_xlfn.XLOOKUP(TRUE, EXACT(G16, Table1[orig]), Table1[(Y)])</f>
+        <v>T2</v>
+      </c>
+      <c r="G16" t="str" cm="1">
+        <f t="array" ref="G16">_xlfn.XLOOKUP(TRUE, EXACT(A16, Table1[orig]), Table1[(Y)])</f>
+        <v>S2</v>
+      </c>
+      <c r="H16" t="str" cm="1">
+        <f t="array" ref="H16">_xlfn.XLOOKUP(TRUE, EXACT(I16, Table3[orig]), Table3[(Z)])</f>
+        <v>H2</v>
+      </c>
+      <c r="I16" t="str" cm="1">
+        <f t="array" ref="I16">_xlfn.XLOOKUP(TRUE, EXACT(J16, Table3[orig]), Table3[(Z)])</f>
+        <v>T2</v>
+      </c>
+      <c r="J16" t="str" cm="1">
+        <f t="array" ref="J16">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>H2</v>
+      </c>
+      <c r="K16" t="str" cm="1">
+        <f t="array" ref="K16">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>T2</v>
+      </c>
+      <c r="L16" t="str" cm="1">
+        <f t="array" ref="L16">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>T2</v>
+      </c>
+      <c r="M16" t="str" cm="1">
+        <f t="array" ref="M16">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>T2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A17" t="str">
+        <f>intermediate!E20</f>
+        <v>l2</v>
+      </c>
+      <c r="B17" t="str" cm="1">
+        <f t="array" ref="B17">_xlfn.XLOOKUP(TRUE, EXACT(C17, Table4[orig]), Table4[(X)])</f>
+        <v>l2</v>
+      </c>
+      <c r="C17" t="str" cm="1">
+        <f t="array" ref="C17">_xlfn.XLOOKUP(TRUE, EXACT(D17, Table4[orig]), Table4[(X)])</f>
+        <v>l2</v>
+      </c>
+      <c r="D17" t="str" cm="1">
+        <f t="array" ref="D17">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>l2</v>
+      </c>
+      <c r="E17" t="str" cm="1">
+        <f t="array" ref="E17">_xlfn.XLOOKUP(TRUE, EXACT(F17, Table1[orig]), Table1[(Y)])</f>
+        <v>f2</v>
+      </c>
+      <c r="F17" t="str" cm="1">
+        <f t="array" ref="F17">_xlfn.XLOOKUP(TRUE, EXACT(G17, Table1[orig]), Table1[(Y)])</f>
+        <v>r2</v>
+      </c>
+      <c r="G17" t="str" cm="1">
+        <f t="array" ref="G17">_xlfn.XLOOKUP(TRUE, EXACT(A17, Table1[orig]), Table1[(Y)])</f>
+        <v>b2</v>
+      </c>
+      <c r="H17" t="str" cm="1">
+        <f t="array" ref="H17">_xlfn.XLOOKUP(TRUE, EXACT(I17, Table3[orig]), Table3[(Z)])</f>
+        <v>d2</v>
+      </c>
+      <c r="I17" t="str" cm="1">
+        <f t="array" ref="I17">_xlfn.XLOOKUP(TRUE, EXACT(J17, Table3[orig]), Table3[(Z)])</f>
+        <v>r2</v>
+      </c>
+      <c r="J17" t="str" cm="1">
+        <f t="array" ref="J17">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>u2</v>
+      </c>
+      <c r="K17" t="str" cm="1">
+        <f t="array" ref="K17">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>r2</v>
+      </c>
+      <c r="L17" t="str" cm="1">
+        <f t="array" ref="L17">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>l2</v>
+      </c>
+      <c r="M17" t="str" cm="1">
+        <f t="array" ref="M17">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>l2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A18" t="str">
+        <f>intermediate!E21</f>
+        <v>L2</v>
+      </c>
+      <c r="B18" t="str" cm="1">
+        <f t="array" ref="B18">_xlfn.XLOOKUP(TRUE, EXACT(C18, Table4[orig]), Table4[(X)])</f>
+        <v>L2</v>
+      </c>
+      <c r="C18" t="str" cm="1">
+        <f t="array" ref="C18">_xlfn.XLOOKUP(TRUE, EXACT(D18, Table4[orig]), Table4[(X)])</f>
+        <v>L2</v>
+      </c>
+      <c r="D18" t="str" cm="1">
+        <f t="array" ref="D18">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>L2</v>
+      </c>
+      <c r="E18" t="str" cm="1">
+        <f t="array" ref="E18">_xlfn.XLOOKUP(TRUE, EXACT(F18, Table1[orig]), Table1[(Y)])</f>
+        <v>F2</v>
+      </c>
+      <c r="F18" t="str" cm="1">
+        <f t="array" ref="F18">_xlfn.XLOOKUP(TRUE, EXACT(G18, Table1[orig]), Table1[(Y)])</f>
+        <v>R2</v>
+      </c>
+      <c r="G18" t="str" cm="1">
+        <f t="array" ref="G18">_xlfn.XLOOKUP(TRUE, EXACT(A18, Table1[orig]), Table1[(Y)])</f>
+        <v>B2</v>
+      </c>
+      <c r="H18" t="str" cm="1">
+        <f t="array" ref="H18">_xlfn.XLOOKUP(TRUE, EXACT(I18, Table3[orig]), Table3[(Z)])</f>
+        <v>D2</v>
+      </c>
+      <c r="I18" t="str" cm="1">
+        <f t="array" ref="I18">_xlfn.XLOOKUP(TRUE, EXACT(J18, Table3[orig]), Table3[(Z)])</f>
+        <v>R2</v>
+      </c>
+      <c r="J18" t="str" cm="1">
+        <f t="array" ref="J18">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>U2</v>
+      </c>
+      <c r="K18" t="str" cm="1">
+        <f t="array" ref="K18">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>R2</v>
+      </c>
+      <c r="L18" t="str" cm="1">
+        <f t="array" ref="L18">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>L2</v>
+      </c>
+      <c r="M18" t="str" cm="1">
+        <f t="array" ref="M18">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>L2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="str">
+        <f>intermediate!E22</f>
+        <v>X2</v>
+      </c>
+      <c r="B19" s="3" t="str" cm="1">
+        <f t="array" ref="B19">_xlfn.XLOOKUP(TRUE, EXACT(C19, Table4[orig]), Table4[(X)])</f>
+        <v>X2</v>
+      </c>
+      <c r="C19" s="3" t="str" cm="1">
+        <f t="array" ref="C19">_xlfn.XLOOKUP(TRUE, EXACT(D19, Table4[orig]), Table4[(X)])</f>
+        <v>X2</v>
+      </c>
+      <c r="D19" s="3" t="str" cm="1">
+        <f t="array" ref="D19">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>X2</v>
+      </c>
+      <c r="E19" s="3" t="str" cm="1">
+        <f t="array" ref="E19">_xlfn.XLOOKUP(TRUE, EXACT(F19, Table1[orig]), Table1[(Y)])</f>
+        <v>Z2</v>
+      </c>
+      <c r="F19" s="3" t="str" cm="1">
+        <f t="array" ref="F19">_xlfn.XLOOKUP(TRUE, EXACT(G19, Table1[orig]), Table1[(Y)])</f>
+        <v>X2</v>
+      </c>
+      <c r="G19" s="3" t="str" cm="1">
+        <f t="array" ref="G19">_xlfn.XLOOKUP(TRUE, EXACT(A19, Table1[orig]), Table1[(Y)])</f>
+        <v>Z2</v>
+      </c>
+      <c r="H19" s="3" t="str" cm="1">
+        <f t="array" ref="H19">_xlfn.XLOOKUP(TRUE, EXACT(I19, Table3[orig]), Table3[(Z)])</f>
+        <v>Y2</v>
+      </c>
+      <c r="I19" s="3" t="str" cm="1">
+        <f t="array" ref="I19">_xlfn.XLOOKUP(TRUE, EXACT(J19, Table3[orig]), Table3[(Z)])</f>
+        <v>X2</v>
+      </c>
+      <c r="J19" s="3" t="str" cm="1">
+        <f t="array" ref="J19">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>Y2</v>
+      </c>
+      <c r="K19" s="3" t="str" cm="1">
+        <f t="array" ref="K19">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>X2</v>
+      </c>
+      <c r="L19" s="3" t="str" cm="1">
+        <f t="array" ref="L19">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>X2</v>
+      </c>
+      <c r="M19" s="3" t="str" cm="1">
+        <f t="array" ref="M19">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>X2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A20" t="str">
+        <f>intermediate!E23</f>
+        <v>F</v>
+      </c>
+      <c r="B20" t="str" cm="1">
+        <f t="array" ref="B20">_xlfn.XLOOKUP(TRUE, EXACT(C20, Table4[orig]), Table4[(X)])</f>
+        <v>D</v>
+      </c>
+      <c r="C20" t="str" cm="1">
+        <f t="array" ref="C20">_xlfn.XLOOKUP(TRUE, EXACT(D20, Table4[orig]), Table4[(X)])</f>
+        <v>B</v>
+      </c>
+      <c r="D20" t="str" cm="1">
+        <f t="array" ref="D20">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>U</v>
+      </c>
+      <c r="E20" t="str" cm="1">
+        <f t="array" ref="E20">_xlfn.XLOOKUP(TRUE, EXACT(F20, Table1[orig]), Table1[(Y)])</f>
+        <v>R</v>
+      </c>
+      <c r="F20" t="str" cm="1">
+        <f t="array" ref="F20">_xlfn.XLOOKUP(TRUE, EXACT(G20, Table1[orig]), Table1[(Y)])</f>
+        <v>B</v>
+      </c>
+      <c r="G20" t="str" cm="1">
+        <f t="array" ref="G20">_xlfn.XLOOKUP(TRUE, EXACT(A20, Table1[orig]), Table1[(Y)])</f>
+        <v>L</v>
+      </c>
+      <c r="H20" t="str" cm="1">
+        <f t="array" ref="H20">_xlfn.XLOOKUP(TRUE, EXACT(I20, Table3[orig]), Table3[(Z)])</f>
+        <v>F</v>
+      </c>
+      <c r="I20" t="str" cm="1">
+        <f t="array" ref="I20">_xlfn.XLOOKUP(TRUE, EXACT(J20, Table3[orig]), Table3[(Z)])</f>
+        <v>F</v>
+      </c>
+      <c r="J20" t="str" cm="1">
+        <f t="array" ref="J20">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>F</v>
+      </c>
+      <c r="K20" t="str" cm="1">
+        <f t="array" ref="K20">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>F'</v>
+      </c>
+      <c r="L20" t="str" cm="1">
+        <f t="array" ref="L20">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>F'</v>
+      </c>
+      <c r="M20" t="str" cm="1">
+        <f t="array" ref="M20">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>B'</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A21" t="str">
+        <f>intermediate!E24</f>
+        <v>f</v>
+      </c>
+      <c r="B21" t="str" cm="1">
+        <f t="array" ref="B21">_xlfn.XLOOKUP(TRUE, EXACT(C21, Table4[orig]), Table4[(X)])</f>
+        <v>d</v>
+      </c>
+      <c r="C21" t="str" cm="1">
+        <f t="array" ref="C21">_xlfn.XLOOKUP(TRUE, EXACT(D21, Table4[orig]), Table4[(X)])</f>
+        <v>b</v>
+      </c>
+      <c r="D21" t="str" cm="1">
+        <f t="array" ref="D21">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>u</v>
+      </c>
+      <c r="E21" t="str" cm="1">
+        <f t="array" ref="E21">_xlfn.XLOOKUP(TRUE, EXACT(F21, Table1[orig]), Table1[(Y)])</f>
+        <v>r</v>
+      </c>
+      <c r="F21" t="str" cm="1">
+        <f t="array" ref="F21">_xlfn.XLOOKUP(TRUE, EXACT(G21, Table1[orig]), Table1[(Y)])</f>
+        <v>b</v>
+      </c>
+      <c r="G21" t="str" cm="1">
+        <f t="array" ref="G21">_xlfn.XLOOKUP(TRUE, EXACT(A21, Table1[orig]), Table1[(Y)])</f>
+        <v>l</v>
+      </c>
+      <c r="H21" t="str" cm="1">
+        <f t="array" ref="H21">_xlfn.XLOOKUP(TRUE, EXACT(I21, Table3[orig]), Table3[(Z)])</f>
+        <v>f</v>
+      </c>
+      <c r="I21" t="str" cm="1">
+        <f t="array" ref="I21">_xlfn.XLOOKUP(TRUE, EXACT(J21, Table3[orig]), Table3[(Z)])</f>
+        <v>f</v>
+      </c>
+      <c r="J21" t="str" cm="1">
+        <f t="array" ref="J21">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>f</v>
+      </c>
+      <c r="K21" t="str" cm="1">
+        <f t="array" ref="K21">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>f'</v>
+      </c>
+      <c r="L21" t="str" cm="1">
+        <f t="array" ref="L21">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>f'</v>
+      </c>
+      <c r="M21" t="str" cm="1">
+        <f t="array" ref="M21">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>b'</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A22" t="str">
+        <f>intermediate!E25</f>
+        <v>S</v>
+      </c>
+      <c r="B22" t="str" cm="1">
+        <f t="array" ref="B22">_xlfn.XLOOKUP(TRUE, EXACT(C22, Table4[orig]), Table4[(X)])</f>
+        <v>H'</v>
+      </c>
+      <c r="C22" t="str" cm="1">
+        <f t="array" ref="C22">_xlfn.XLOOKUP(TRUE, EXACT(D22, Table4[orig]), Table4[(X)])</f>
+        <v>S'</v>
+      </c>
+      <c r="D22" t="str" cm="1">
+        <f t="array" ref="D22">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>H</v>
+      </c>
+      <c r="E22" t="str" cm="1">
+        <f t="array" ref="E22">_xlfn.XLOOKUP(TRUE, EXACT(F22, Table1[orig]), Table1[(Y)])</f>
+        <v>T</v>
+      </c>
+      <c r="F22" t="str" cm="1">
+        <f t="array" ref="F22">_xlfn.XLOOKUP(TRUE, EXACT(G22, Table1[orig]), Table1[(Y)])</f>
+        <v>S'</v>
+      </c>
+      <c r="G22" t="str" cm="1">
+        <f t="array" ref="G22">_xlfn.XLOOKUP(TRUE, EXACT(A22, Table1[orig]), Table1[(Y)])</f>
+        <v>T'</v>
+      </c>
+      <c r="H22" t="str" cm="1">
+        <f t="array" ref="H22">_xlfn.XLOOKUP(TRUE, EXACT(I22, Table3[orig]), Table3[(Z)])</f>
+        <v>S</v>
+      </c>
+      <c r="I22" t="str" cm="1">
+        <f t="array" ref="I22">_xlfn.XLOOKUP(TRUE, EXACT(J22, Table3[orig]), Table3[(Z)])</f>
+        <v>S</v>
+      </c>
+      <c r="J22" t="str" cm="1">
+        <f t="array" ref="J22">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>S</v>
+      </c>
+      <c r="K22" t="str" cm="1">
+        <f t="array" ref="K22">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>S'</v>
+      </c>
+      <c r="L22" t="str" cm="1">
+        <f t="array" ref="L22">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>S'</v>
+      </c>
+      <c r="M22" t="str" cm="1">
+        <f t="array" ref="M22">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>S</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A23" t="str">
+        <f>intermediate!E26</f>
+        <v>b</v>
+      </c>
+      <c r="B23" t="str" cm="1">
+        <f t="array" ref="B23">_xlfn.XLOOKUP(TRUE, EXACT(C23, Table4[orig]), Table4[(X)])</f>
+        <v>u</v>
+      </c>
+      <c r="C23" t="str" cm="1">
+        <f t="array" ref="C23">_xlfn.XLOOKUP(TRUE, EXACT(D23, Table4[orig]), Table4[(X)])</f>
+        <v>f</v>
+      </c>
+      <c r="D23" t="str" cm="1">
+        <f t="array" ref="D23">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>d</v>
+      </c>
+      <c r="E23" t="str" cm="1">
+        <f t="array" ref="E23">_xlfn.XLOOKUP(TRUE, EXACT(F23, Table1[orig]), Table1[(Y)])</f>
+        <v>l</v>
+      </c>
+      <c r="F23" t="str" cm="1">
+        <f t="array" ref="F23">_xlfn.XLOOKUP(TRUE, EXACT(G23, Table1[orig]), Table1[(Y)])</f>
+        <v>f</v>
+      </c>
+      <c r="G23" t="str" cm="1">
+        <f t="array" ref="G23">_xlfn.XLOOKUP(TRUE, EXACT(A23, Table1[orig]), Table1[(Y)])</f>
+        <v>r</v>
+      </c>
+      <c r="H23" t="str" cm="1">
+        <f t="array" ref="H23">_xlfn.XLOOKUP(TRUE, EXACT(I23, Table3[orig]), Table3[(Z)])</f>
+        <v>b</v>
+      </c>
+      <c r="I23" t="str" cm="1">
+        <f t="array" ref="I23">_xlfn.XLOOKUP(TRUE, EXACT(J23, Table3[orig]), Table3[(Z)])</f>
+        <v>b</v>
+      </c>
+      <c r="J23" t="str" cm="1">
+        <f t="array" ref="J23">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>b</v>
+      </c>
+      <c r="K23" t="str" cm="1">
+        <f t="array" ref="K23">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>b'</v>
+      </c>
+      <c r="L23" t="str" cm="1">
+        <f t="array" ref="L23">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>b'</v>
+      </c>
+      <c r="M23" t="str" cm="1">
+        <f t="array" ref="M23">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>f'</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A24" t="str">
+        <f>intermediate!E27</f>
+        <v>B</v>
+      </c>
+      <c r="B24" t="str" cm="1">
+        <f t="array" ref="B24">_xlfn.XLOOKUP(TRUE, EXACT(C24, Table4[orig]), Table4[(X)])</f>
+        <v>U</v>
+      </c>
+      <c r="C24" t="str" cm="1">
+        <f t="array" ref="C24">_xlfn.XLOOKUP(TRUE, EXACT(D24, Table4[orig]), Table4[(X)])</f>
+        <v>F</v>
+      </c>
+      <c r="D24" t="str" cm="1">
+        <f t="array" ref="D24">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>D</v>
+      </c>
+      <c r="E24" t="str" cm="1">
+        <f t="array" ref="E24">_xlfn.XLOOKUP(TRUE, EXACT(F24, Table1[orig]), Table1[(Y)])</f>
+        <v>L</v>
+      </c>
+      <c r="F24" t="str" cm="1">
+        <f t="array" ref="F24">_xlfn.XLOOKUP(TRUE, EXACT(G24, Table1[orig]), Table1[(Y)])</f>
+        <v>F</v>
+      </c>
+      <c r="G24" t="str" cm="1">
+        <f t="array" ref="G24">_xlfn.XLOOKUP(TRUE, EXACT(A24, Table1[orig]), Table1[(Y)])</f>
+        <v>R</v>
+      </c>
+      <c r="H24" t="str" cm="1">
+        <f t="array" ref="H24">_xlfn.XLOOKUP(TRUE, EXACT(I24, Table3[orig]), Table3[(Z)])</f>
+        <v>B</v>
+      </c>
+      <c r="I24" t="str" cm="1">
+        <f t="array" ref="I24">_xlfn.XLOOKUP(TRUE, EXACT(J24, Table3[orig]), Table3[(Z)])</f>
+        <v>B</v>
+      </c>
+      <c r="J24" t="str" cm="1">
+        <f t="array" ref="J24">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>B</v>
+      </c>
+      <c r="K24" t="str" cm="1">
+        <f t="array" ref="K24">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>B'</v>
+      </c>
+      <c r="L24" t="str" cm="1">
+        <f t="array" ref="L24">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>B'</v>
+      </c>
+      <c r="M24" t="str" cm="1">
+        <f t="array" ref="M24">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>F'</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="str">
+        <f>intermediate!E28</f>
+        <v>Z</v>
+      </c>
+      <c r="B25" s="3" t="str" cm="1">
+        <f t="array" ref="B25">_xlfn.XLOOKUP(TRUE, EXACT(C25, Table4[orig]), Table4[(X)])</f>
+        <v>Y'</v>
+      </c>
+      <c r="C25" s="3" t="str" cm="1">
+        <f t="array" ref="C25">_xlfn.XLOOKUP(TRUE, EXACT(D25, Table4[orig]), Table4[(X)])</f>
+        <v>Z'</v>
+      </c>
+      <c r="D25" s="3" t="str" cm="1">
+        <f t="array" ref="D25">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>Y</v>
+      </c>
+      <c r="E25" s="3" t="str" cm="1">
+        <f t="array" ref="E25">_xlfn.XLOOKUP(TRUE, EXACT(F25, Table1[orig]), Table1[(Y)])</f>
+        <v>X</v>
+      </c>
+      <c r="F25" s="3" t="str" cm="1">
+        <f t="array" ref="F25">_xlfn.XLOOKUP(TRUE, EXACT(G25, Table1[orig]), Table1[(Y)])</f>
+        <v>Z'</v>
+      </c>
+      <c r="G25" s="3" t="str" cm="1">
+        <f t="array" ref="G25">_xlfn.XLOOKUP(TRUE, EXACT(A25, Table1[orig]), Table1[(Y)])</f>
+        <v>X'</v>
+      </c>
+      <c r="H25" s="3" t="str" cm="1">
+        <f t="array" ref="H25">_xlfn.XLOOKUP(TRUE, EXACT(I25, Table3[orig]), Table3[(Z)])</f>
+        <v>Z</v>
+      </c>
+      <c r="I25" s="3" t="str" cm="1">
+        <f t="array" ref="I25">_xlfn.XLOOKUP(TRUE, EXACT(J25, Table3[orig]), Table3[(Z)])</f>
+        <v>Z</v>
+      </c>
+      <c r="J25" s="3" t="str" cm="1">
+        <f t="array" ref="J25">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>Z</v>
+      </c>
+      <c r="K25" s="3" t="str" cm="1">
+        <f t="array" ref="K25">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>Z'</v>
+      </c>
+      <c r="L25" s="3" t="str" cm="1">
+        <f t="array" ref="L25">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>Z'</v>
+      </c>
+      <c r="M25" s="3" t="str" cm="1">
+        <f t="array" ref="M25">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>Z</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A26" t="str">
+        <f>intermediate!E29</f>
+        <v>F'</v>
+      </c>
+      <c r="B26" t="str" cm="1">
+        <f t="array" ref="B26">_xlfn.XLOOKUP(TRUE, EXACT(C26, Table4[orig]), Table4[(X)])</f>
+        <v>D'</v>
+      </c>
+      <c r="C26" t="str" cm="1">
+        <f t="array" ref="C26">_xlfn.XLOOKUP(TRUE, EXACT(D26, Table4[orig]), Table4[(X)])</f>
+        <v>B'</v>
+      </c>
+      <c r="D26" t="str" cm="1">
+        <f t="array" ref="D26">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>U'</v>
+      </c>
+      <c r="E26" t="str" cm="1">
+        <f t="array" ref="E26">_xlfn.XLOOKUP(TRUE, EXACT(F26, Table1[orig]), Table1[(Y)])</f>
+        <v>R'</v>
+      </c>
+      <c r="F26" t="str" cm="1">
+        <f t="array" ref="F26">_xlfn.XLOOKUP(TRUE, EXACT(G26, Table1[orig]), Table1[(Y)])</f>
+        <v>B'</v>
+      </c>
+      <c r="G26" t="str" cm="1">
+        <f t="array" ref="G26">_xlfn.XLOOKUP(TRUE, EXACT(A26, Table1[orig]), Table1[(Y)])</f>
+        <v>L'</v>
+      </c>
+      <c r="H26" t="str" cm="1">
+        <f t="array" ref="H26">_xlfn.XLOOKUP(TRUE, EXACT(I26, Table3[orig]), Table3[(Z)])</f>
+        <v>F'</v>
+      </c>
+      <c r="I26" t="str" cm="1">
+        <f t="array" ref="I26">_xlfn.XLOOKUP(TRUE, EXACT(J26, Table3[orig]), Table3[(Z)])</f>
+        <v>F'</v>
+      </c>
+      <c r="J26" t="str" cm="1">
+        <f t="array" ref="J26">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>F'</v>
+      </c>
+      <c r="K26" t="str" cm="1">
+        <f t="array" ref="K26">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>F</v>
+      </c>
+      <c r="L26" t="str" cm="1">
+        <f t="array" ref="L26">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>F</v>
+      </c>
+      <c r="M26" t="str" cm="1">
+        <f t="array" ref="M26">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A27" t="str">
+        <f>intermediate!E30</f>
+        <v>f'</v>
+      </c>
+      <c r="B27" t="str" cm="1">
+        <f t="array" ref="B27">_xlfn.XLOOKUP(TRUE, EXACT(C27, Table4[orig]), Table4[(X)])</f>
+        <v>d'</v>
+      </c>
+      <c r="C27" t="str" cm="1">
+        <f t="array" ref="C27">_xlfn.XLOOKUP(TRUE, EXACT(D27, Table4[orig]), Table4[(X)])</f>
+        <v>b'</v>
+      </c>
+      <c r="D27" t="str" cm="1">
+        <f t="array" ref="D27">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>u'</v>
+      </c>
+      <c r="E27" t="str" cm="1">
+        <f t="array" ref="E27">_xlfn.XLOOKUP(TRUE, EXACT(F27, Table1[orig]), Table1[(Y)])</f>
+        <v>r'</v>
+      </c>
+      <c r="F27" t="str" cm="1">
+        <f t="array" ref="F27">_xlfn.XLOOKUP(TRUE, EXACT(G27, Table1[orig]), Table1[(Y)])</f>
+        <v>b'</v>
+      </c>
+      <c r="G27" t="str" cm="1">
+        <f t="array" ref="G27">_xlfn.XLOOKUP(TRUE, EXACT(A27, Table1[orig]), Table1[(Y)])</f>
+        <v>l'</v>
+      </c>
+      <c r="H27" t="str" cm="1">
+        <f t="array" ref="H27">_xlfn.XLOOKUP(TRUE, EXACT(I27, Table3[orig]), Table3[(Z)])</f>
+        <v>f'</v>
+      </c>
+      <c r="I27" t="str" cm="1">
+        <f t="array" ref="I27">_xlfn.XLOOKUP(TRUE, EXACT(J27, Table3[orig]), Table3[(Z)])</f>
+        <v>f'</v>
+      </c>
+      <c r="J27" t="str" cm="1">
+        <f t="array" ref="J27">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>f'</v>
+      </c>
+      <c r="K27" t="str" cm="1">
+        <f t="array" ref="K27">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>f</v>
+      </c>
+      <c r="L27" t="str" cm="1">
+        <f t="array" ref="L27">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>f</v>
+      </c>
+      <c r="M27" t="str" cm="1">
+        <f t="array" ref="M27">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>b</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A28" t="str">
+        <f>intermediate!E31</f>
+        <v>S'</v>
+      </c>
+      <c r="B28" t="str" cm="1">
+        <f t="array" ref="B28">_xlfn.XLOOKUP(TRUE, EXACT(C28, Table4[orig]), Table4[(X)])</f>
+        <v>H</v>
+      </c>
+      <c r="C28" t="str" cm="1">
+        <f t="array" ref="C28">_xlfn.XLOOKUP(TRUE, EXACT(D28, Table4[orig]), Table4[(X)])</f>
+        <v>S</v>
+      </c>
+      <c r="D28" t="str" cm="1">
+        <f t="array" ref="D28">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>H'</v>
+      </c>
+      <c r="E28" t="str" cm="1">
+        <f t="array" ref="E28">_xlfn.XLOOKUP(TRUE, EXACT(F28, Table1[orig]), Table1[(Y)])</f>
+        <v>T'</v>
+      </c>
+      <c r="F28" t="str" cm="1">
+        <f t="array" ref="F28">_xlfn.XLOOKUP(TRUE, EXACT(G28, Table1[orig]), Table1[(Y)])</f>
+        <v>S</v>
+      </c>
+      <c r="G28" t="str" cm="1">
+        <f t="array" ref="G28">_xlfn.XLOOKUP(TRUE, EXACT(A28, Table1[orig]), Table1[(Y)])</f>
+        <v>T</v>
+      </c>
+      <c r="H28" t="str" cm="1">
+        <f t="array" ref="H28">_xlfn.XLOOKUP(TRUE, EXACT(I28, Table3[orig]), Table3[(Z)])</f>
+        <v>S'</v>
+      </c>
+      <c r="I28" t="str" cm="1">
+        <f t="array" ref="I28">_xlfn.XLOOKUP(TRUE, EXACT(J28, Table3[orig]), Table3[(Z)])</f>
+        <v>S'</v>
+      </c>
+      <c r="J28" t="str" cm="1">
+        <f t="array" ref="J28">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>S'</v>
+      </c>
+      <c r="K28" t="str" cm="1">
+        <f t="array" ref="K28">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>S</v>
+      </c>
+      <c r="L28" t="str" cm="1">
+        <f t="array" ref="L28">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>S</v>
+      </c>
+      <c r="M28" t="str" cm="1">
+        <f t="array" ref="M28">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>S'</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A29" t="str">
+        <f>intermediate!E32</f>
+        <v>b'</v>
+      </c>
+      <c r="B29" t="str" cm="1">
+        <f t="array" ref="B29">_xlfn.XLOOKUP(TRUE, EXACT(C29, Table4[orig]), Table4[(X)])</f>
+        <v>u'</v>
+      </c>
+      <c r="C29" t="str" cm="1">
+        <f t="array" ref="C29">_xlfn.XLOOKUP(TRUE, EXACT(D29, Table4[orig]), Table4[(X)])</f>
+        <v>f'</v>
+      </c>
+      <c r="D29" t="str" cm="1">
+        <f t="array" ref="D29">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>d'</v>
+      </c>
+      <c r="E29" t="str" cm="1">
+        <f t="array" ref="E29">_xlfn.XLOOKUP(TRUE, EXACT(F29, Table1[orig]), Table1[(Y)])</f>
+        <v>l'</v>
+      </c>
+      <c r="F29" t="str" cm="1">
+        <f t="array" ref="F29">_xlfn.XLOOKUP(TRUE, EXACT(G29, Table1[orig]), Table1[(Y)])</f>
+        <v>f'</v>
+      </c>
+      <c r="G29" t="str" cm="1">
+        <f t="array" ref="G29">_xlfn.XLOOKUP(TRUE, EXACT(A29, Table1[orig]), Table1[(Y)])</f>
+        <v>r'</v>
+      </c>
+      <c r="H29" t="str" cm="1">
+        <f t="array" ref="H29">_xlfn.XLOOKUP(TRUE, EXACT(I29, Table3[orig]), Table3[(Z)])</f>
+        <v>b'</v>
+      </c>
+      <c r="I29" t="str" cm="1">
+        <f t="array" ref="I29">_xlfn.XLOOKUP(TRUE, EXACT(J29, Table3[orig]), Table3[(Z)])</f>
+        <v>b'</v>
+      </c>
+      <c r="J29" t="str" cm="1">
+        <f t="array" ref="J29">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>b'</v>
+      </c>
+      <c r="K29" t="str" cm="1">
+        <f t="array" ref="K29">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>b</v>
+      </c>
+      <c r="L29" t="str" cm="1">
+        <f t="array" ref="L29">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>b</v>
+      </c>
+      <c r="M29" t="str" cm="1">
+        <f t="array" ref="M29">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>f</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A30" t="str">
+        <f>intermediate!E33</f>
+        <v>B'</v>
+      </c>
+      <c r="B30" t="str" cm="1">
+        <f t="array" ref="B30">_xlfn.XLOOKUP(TRUE, EXACT(C30, Table4[orig]), Table4[(X)])</f>
+        <v>U'</v>
+      </c>
+      <c r="C30" t="str" cm="1">
+        <f t="array" ref="C30">_xlfn.XLOOKUP(TRUE, EXACT(D30, Table4[orig]), Table4[(X)])</f>
+        <v>F'</v>
+      </c>
+      <c r="D30" t="str" cm="1">
+        <f t="array" ref="D30">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>D'</v>
+      </c>
+      <c r="E30" t="str" cm="1">
+        <f t="array" ref="E30">_xlfn.XLOOKUP(TRUE, EXACT(F30, Table1[orig]), Table1[(Y)])</f>
+        <v>L'</v>
+      </c>
+      <c r="F30" t="str" cm="1">
+        <f t="array" ref="F30">_xlfn.XLOOKUP(TRUE, EXACT(G30, Table1[orig]), Table1[(Y)])</f>
+        <v>F'</v>
+      </c>
+      <c r="G30" t="str" cm="1">
+        <f t="array" ref="G30">_xlfn.XLOOKUP(TRUE, EXACT(A30, Table1[orig]), Table1[(Y)])</f>
+        <v>R'</v>
+      </c>
+      <c r="H30" t="str" cm="1">
+        <f t="array" ref="H30">_xlfn.XLOOKUP(TRUE, EXACT(I30, Table3[orig]), Table3[(Z)])</f>
+        <v>B'</v>
+      </c>
+      <c r="I30" t="str" cm="1">
+        <f t="array" ref="I30">_xlfn.XLOOKUP(TRUE, EXACT(J30, Table3[orig]), Table3[(Z)])</f>
+        <v>B'</v>
+      </c>
+      <c r="J30" t="str" cm="1">
+        <f t="array" ref="J30">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>B'</v>
+      </c>
+      <c r="K30" t="str" cm="1">
+        <f t="array" ref="K30">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>B</v>
+      </c>
+      <c r="L30" t="str" cm="1">
+        <f t="array" ref="L30">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>B</v>
+      </c>
+      <c r="M30" t="str" cm="1">
+        <f t="array" ref="M30">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>F</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A31" s="3" t="str">
+        <f>intermediate!E34</f>
+        <v>Z'</v>
+      </c>
+      <c r="B31" s="3" t="str" cm="1">
+        <f t="array" ref="B31">_xlfn.XLOOKUP(TRUE, EXACT(C31, Table4[orig]), Table4[(X)])</f>
+        <v>Y</v>
+      </c>
+      <c r="C31" s="3" t="str" cm="1">
+        <f t="array" ref="C31">_xlfn.XLOOKUP(TRUE, EXACT(D31, Table4[orig]), Table4[(X)])</f>
+        <v>Z</v>
+      </c>
+      <c r="D31" s="3" t="str" cm="1">
+        <f t="array" ref="D31">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>Y'</v>
+      </c>
+      <c r="E31" s="3" t="str" cm="1">
+        <f t="array" ref="E31">_xlfn.XLOOKUP(TRUE, EXACT(F31, Table1[orig]), Table1[(Y)])</f>
+        <v>X'</v>
+      </c>
+      <c r="F31" s="3" t="str" cm="1">
+        <f t="array" ref="F31">_xlfn.XLOOKUP(TRUE, EXACT(G31, Table1[orig]), Table1[(Y)])</f>
+        <v>Z</v>
+      </c>
+      <c r="G31" s="3" t="str" cm="1">
+        <f t="array" ref="G31">_xlfn.XLOOKUP(TRUE, EXACT(A31, Table1[orig]), Table1[(Y)])</f>
+        <v>X</v>
+      </c>
+      <c r="H31" s="3" t="str" cm="1">
+        <f t="array" ref="H31">_xlfn.XLOOKUP(TRUE, EXACT(I31, Table3[orig]), Table3[(Z)])</f>
+        <v>Z'</v>
+      </c>
+      <c r="I31" s="3" t="str" cm="1">
+        <f t="array" ref="I31">_xlfn.XLOOKUP(TRUE, EXACT(J31, Table3[orig]), Table3[(Z)])</f>
+        <v>Z'</v>
+      </c>
+      <c r="J31" s="3" t="str" cm="1">
+        <f t="array" ref="J31">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>Z'</v>
+      </c>
+      <c r="K31" s="3" t="str" cm="1">
+        <f t="array" ref="K31">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>Z</v>
+      </c>
+      <c r="L31" s="3" t="str" cm="1">
+        <f t="array" ref="L31">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>Z</v>
+      </c>
+      <c r="M31" s="3" t="str" cm="1">
+        <f t="array" ref="M31">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>Z'</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A32" t="str">
+        <f>intermediate!E35</f>
+        <v>F2</v>
+      </c>
+      <c r="B32" t="str" cm="1">
+        <f t="array" ref="B32">_xlfn.XLOOKUP(TRUE, EXACT(C32, Table4[orig]), Table4[(X)])</f>
+        <v>D2</v>
+      </c>
+      <c r="C32" t="str" cm="1">
+        <f t="array" ref="C32">_xlfn.XLOOKUP(TRUE, EXACT(D32, Table4[orig]), Table4[(X)])</f>
+        <v>B2</v>
+      </c>
+      <c r="D32" t="str" cm="1">
+        <f t="array" ref="D32">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>U2</v>
+      </c>
+      <c r="E32" t="str" cm="1">
+        <f t="array" ref="E32">_xlfn.XLOOKUP(TRUE, EXACT(F32, Table1[orig]), Table1[(Y)])</f>
+        <v>R2</v>
+      </c>
+      <c r="F32" t="str" cm="1">
+        <f t="array" ref="F32">_xlfn.XLOOKUP(TRUE, EXACT(G32, Table1[orig]), Table1[(Y)])</f>
+        <v>B2</v>
+      </c>
+      <c r="G32" t="str" cm="1">
+        <f t="array" ref="G32">_xlfn.XLOOKUP(TRUE, EXACT(A32, Table1[orig]), Table1[(Y)])</f>
+        <v>L2</v>
+      </c>
+      <c r="H32" t="str" cm="1">
+        <f t="array" ref="H32">_xlfn.XLOOKUP(TRUE, EXACT(I32, Table3[orig]), Table3[(Z)])</f>
+        <v>F2</v>
+      </c>
+      <c r="I32" t="str" cm="1">
+        <f t="array" ref="I32">_xlfn.XLOOKUP(TRUE, EXACT(J32, Table3[orig]), Table3[(Z)])</f>
+        <v>F2</v>
+      </c>
+      <c r="J32" t="str" cm="1">
+        <f t="array" ref="J32">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>F2</v>
+      </c>
+      <c r="K32" t="str" cm="1">
+        <f t="array" ref="K32">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>F2</v>
+      </c>
+      <c r="L32" t="str" cm="1">
+        <f t="array" ref="L32">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>F2</v>
+      </c>
+      <c r="M32" t="str" cm="1">
+        <f t="array" ref="M32">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>B2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A33" t="str">
+        <f>intermediate!E36</f>
+        <v>f2</v>
+      </c>
+      <c r="B33" t="str" cm="1">
+        <f t="array" ref="B33">_xlfn.XLOOKUP(TRUE, EXACT(C33, Table4[orig]), Table4[(X)])</f>
+        <v>d2</v>
+      </c>
+      <c r="C33" t="str" cm="1">
+        <f t="array" ref="C33">_xlfn.XLOOKUP(TRUE, EXACT(D33, Table4[orig]), Table4[(X)])</f>
+        <v>b2</v>
+      </c>
+      <c r="D33" t="str" cm="1">
+        <f t="array" ref="D33">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>u2</v>
+      </c>
+      <c r="E33" t="str" cm="1">
+        <f t="array" ref="E33">_xlfn.XLOOKUP(TRUE, EXACT(F33, Table1[orig]), Table1[(Y)])</f>
+        <v>r2</v>
+      </c>
+      <c r="F33" t="str" cm="1">
+        <f t="array" ref="F33">_xlfn.XLOOKUP(TRUE, EXACT(G33, Table1[orig]), Table1[(Y)])</f>
+        <v>b2</v>
+      </c>
+      <c r="G33" t="str" cm="1">
+        <f t="array" ref="G33">_xlfn.XLOOKUP(TRUE, EXACT(A33, Table1[orig]), Table1[(Y)])</f>
+        <v>l2</v>
+      </c>
+      <c r="H33" t="str" cm="1">
+        <f t="array" ref="H33">_xlfn.XLOOKUP(TRUE, EXACT(I33, Table3[orig]), Table3[(Z)])</f>
+        <v>f2</v>
+      </c>
+      <c r="I33" t="str" cm="1">
+        <f t="array" ref="I33">_xlfn.XLOOKUP(TRUE, EXACT(J33, Table3[orig]), Table3[(Z)])</f>
+        <v>f2</v>
+      </c>
+      <c r="J33" t="str" cm="1">
+        <f t="array" ref="J33">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>f2</v>
+      </c>
+      <c r="K33" t="str" cm="1">
+        <f t="array" ref="K33">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>f2</v>
+      </c>
+      <c r="L33" t="str" cm="1">
+        <f t="array" ref="L33">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>f2</v>
+      </c>
+      <c r="M33" t="str" cm="1">
+        <f t="array" ref="M33">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>b2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A34" t="str">
+        <f>intermediate!E37</f>
+        <v>S2</v>
+      </c>
+      <c r="B34" t="str" cm="1">
+        <f t="array" ref="B34">_xlfn.XLOOKUP(TRUE, EXACT(C34, Table4[orig]), Table4[(X)])</f>
+        <v>H2</v>
+      </c>
+      <c r="C34" t="str" cm="1">
+        <f t="array" ref="C34">_xlfn.XLOOKUP(TRUE, EXACT(D34, Table4[orig]), Table4[(X)])</f>
+        <v>S2</v>
+      </c>
+      <c r="D34" t="str" cm="1">
+        <f t="array" ref="D34">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>H2</v>
+      </c>
+      <c r="E34" t="str" cm="1">
+        <f t="array" ref="E34">_xlfn.XLOOKUP(TRUE, EXACT(F34, Table1[orig]), Table1[(Y)])</f>
+        <v>T2</v>
+      </c>
+      <c r="F34" t="str" cm="1">
+        <f t="array" ref="F34">_xlfn.XLOOKUP(TRUE, EXACT(G34, Table1[orig]), Table1[(Y)])</f>
+        <v>S2</v>
+      </c>
+      <c r="G34" t="str" cm="1">
+        <f t="array" ref="G34">_xlfn.XLOOKUP(TRUE, EXACT(A34, Table1[orig]), Table1[(Y)])</f>
+        <v>T2</v>
+      </c>
+      <c r="H34" t="str" cm="1">
+        <f t="array" ref="H34">_xlfn.XLOOKUP(TRUE, EXACT(I34, Table3[orig]), Table3[(Z)])</f>
+        <v>S2</v>
+      </c>
+      <c r="I34" t="str" cm="1">
+        <f t="array" ref="I34">_xlfn.XLOOKUP(TRUE, EXACT(J34, Table3[orig]), Table3[(Z)])</f>
+        <v>S2</v>
+      </c>
+      <c r="J34" t="str" cm="1">
+        <f t="array" ref="J34">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>S2</v>
+      </c>
+      <c r="K34" t="str" cm="1">
+        <f t="array" ref="K34">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>S2</v>
+      </c>
+      <c r="L34" t="str" cm="1">
+        <f t="array" ref="L34">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>S2</v>
+      </c>
+      <c r="M34" t="str" cm="1">
+        <f t="array" ref="M34">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>S2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A35" t="str">
+        <f>intermediate!E38</f>
+        <v>b2</v>
+      </c>
+      <c r="B35" t="str" cm="1">
+        <f t="array" ref="B35">_xlfn.XLOOKUP(TRUE, EXACT(C35, Table4[orig]), Table4[(X)])</f>
+        <v>u2</v>
+      </c>
+      <c r="C35" t="str" cm="1">
+        <f t="array" ref="C35">_xlfn.XLOOKUP(TRUE, EXACT(D35, Table4[orig]), Table4[(X)])</f>
+        <v>f2</v>
+      </c>
+      <c r="D35" t="str" cm="1">
+        <f t="array" ref="D35">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>d2</v>
+      </c>
+      <c r="E35" t="str" cm="1">
+        <f t="array" ref="E35">_xlfn.XLOOKUP(TRUE, EXACT(F35, Table1[orig]), Table1[(Y)])</f>
+        <v>l2</v>
+      </c>
+      <c r="F35" t="str" cm="1">
+        <f t="array" ref="F35">_xlfn.XLOOKUP(TRUE, EXACT(G35, Table1[orig]), Table1[(Y)])</f>
+        <v>f2</v>
+      </c>
+      <c r="G35" t="str" cm="1">
+        <f t="array" ref="G35">_xlfn.XLOOKUP(TRUE, EXACT(A35, Table1[orig]), Table1[(Y)])</f>
+        <v>r2</v>
+      </c>
+      <c r="H35" t="str" cm="1">
+        <f t="array" ref="H35">_xlfn.XLOOKUP(TRUE, EXACT(I35, Table3[orig]), Table3[(Z)])</f>
+        <v>b2</v>
+      </c>
+      <c r="I35" t="str" cm="1">
+        <f t="array" ref="I35">_xlfn.XLOOKUP(TRUE, EXACT(J35, Table3[orig]), Table3[(Z)])</f>
+        <v>b2</v>
+      </c>
+      <c r="J35" t="str" cm="1">
+        <f t="array" ref="J35">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>b2</v>
+      </c>
+      <c r="K35" t="str" cm="1">
+        <f t="array" ref="K35">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>b2</v>
+      </c>
+      <c r="L35" t="str" cm="1">
+        <f t="array" ref="L35">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>b2</v>
+      </c>
+      <c r="M35" t="str" cm="1">
+        <f t="array" ref="M35">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>f2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A36" t="str">
+        <f>intermediate!E39</f>
+        <v>B2</v>
+      </c>
+      <c r="B36" t="str" cm="1">
+        <f t="array" ref="B36">_xlfn.XLOOKUP(TRUE, EXACT(C36, Table4[orig]), Table4[(X)])</f>
+        <v>U2</v>
+      </c>
+      <c r="C36" t="str" cm="1">
+        <f t="array" ref="C36">_xlfn.XLOOKUP(TRUE, EXACT(D36, Table4[orig]), Table4[(X)])</f>
+        <v>F2</v>
+      </c>
+      <c r="D36" t="str" cm="1">
+        <f t="array" ref="D36">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>D2</v>
+      </c>
+      <c r="E36" t="str" cm="1">
+        <f t="array" ref="E36">_xlfn.XLOOKUP(TRUE, EXACT(F36, Table1[orig]), Table1[(Y)])</f>
+        <v>L2</v>
+      </c>
+      <c r="F36" t="str" cm="1">
+        <f t="array" ref="F36">_xlfn.XLOOKUP(TRUE, EXACT(G36, Table1[orig]), Table1[(Y)])</f>
+        <v>F2</v>
+      </c>
+      <c r="G36" t="str" cm="1">
+        <f t="array" ref="G36">_xlfn.XLOOKUP(TRUE, EXACT(A36, Table1[orig]), Table1[(Y)])</f>
+        <v>R2</v>
+      </c>
+      <c r="H36" t="str" cm="1">
+        <f t="array" ref="H36">_xlfn.XLOOKUP(TRUE, EXACT(I36, Table3[orig]), Table3[(Z)])</f>
+        <v>B2</v>
+      </c>
+      <c r="I36" t="str" cm="1">
+        <f t="array" ref="I36">_xlfn.XLOOKUP(TRUE, EXACT(J36, Table3[orig]), Table3[(Z)])</f>
+        <v>B2</v>
+      </c>
+      <c r="J36" t="str" cm="1">
+        <f t="array" ref="J36">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>B2</v>
+      </c>
+      <c r="K36" t="str" cm="1">
+        <f t="array" ref="K36">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>B2</v>
+      </c>
+      <c r="L36" t="str" cm="1">
+        <f t="array" ref="L36">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>B2</v>
+      </c>
+      <c r="M36" t="str" cm="1">
+        <f t="array" ref="M36">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>F2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A37" s="3" t="str">
+        <f>intermediate!E40</f>
+        <v>Z2</v>
+      </c>
+      <c r="B37" s="3" t="str" cm="1">
+        <f t="array" ref="B37">_xlfn.XLOOKUP(TRUE, EXACT(C37, Table4[orig]), Table4[(X)])</f>
+        <v>Y2</v>
+      </c>
+      <c r="C37" s="3" t="str" cm="1">
+        <f t="array" ref="C37">_xlfn.XLOOKUP(TRUE, EXACT(D37, Table4[orig]), Table4[(X)])</f>
+        <v>Z2</v>
+      </c>
+      <c r="D37" s="3" t="str" cm="1">
+        <f t="array" ref="D37">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>Y2</v>
+      </c>
+      <c r="E37" s="3" t="str" cm="1">
+        <f t="array" ref="E37">_xlfn.XLOOKUP(TRUE, EXACT(F37, Table1[orig]), Table1[(Y)])</f>
+        <v>X2</v>
+      </c>
+      <c r="F37" s="3" t="str" cm="1">
+        <f t="array" ref="F37">_xlfn.XLOOKUP(TRUE, EXACT(G37, Table1[orig]), Table1[(Y)])</f>
+        <v>Z2</v>
+      </c>
+      <c r="G37" s="3" t="str" cm="1">
+        <f t="array" ref="G37">_xlfn.XLOOKUP(TRUE, EXACT(A37, Table1[orig]), Table1[(Y)])</f>
+        <v>X2</v>
+      </c>
+      <c r="H37" s="3" t="str" cm="1">
+        <f t="array" ref="H37">_xlfn.XLOOKUP(TRUE, EXACT(I37, Table3[orig]), Table3[(Z)])</f>
+        <v>Z2</v>
+      </c>
+      <c r="I37" s="3" t="str" cm="1">
+        <f t="array" ref="I37">_xlfn.XLOOKUP(TRUE, EXACT(J37, Table3[orig]), Table3[(Z)])</f>
+        <v>Z2</v>
+      </c>
+      <c r="J37" s="3" t="str" cm="1">
+        <f t="array" ref="J37">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>Z2</v>
+      </c>
+      <c r="K37" s="3" t="str" cm="1">
+        <f t="array" ref="K37">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>Z2</v>
+      </c>
+      <c r="L37" s="3" t="str" cm="1">
+        <f t="array" ref="L37">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>Z2</v>
+      </c>
+      <c r="M37" s="3" t="str" cm="1">
+        <f t="array" ref="M37">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>Z2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A38" t="str">
+        <f>intermediate!E41</f>
+        <v>U</v>
+      </c>
+      <c r="B38" t="str" cm="1">
+        <f t="array" ref="B38">_xlfn.XLOOKUP(TRUE, EXACT(C38, Table4[orig]), Table4[(X)])</f>
+        <v>F</v>
+      </c>
+      <c r="C38" t="str" cm="1">
+        <f t="array" ref="C38">_xlfn.XLOOKUP(TRUE, EXACT(D38, Table4[orig]), Table4[(X)])</f>
+        <v>D</v>
+      </c>
+      <c r="D38" t="str" cm="1">
+        <f t="array" ref="D38">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>B</v>
+      </c>
+      <c r="E38" t="str" cm="1">
+        <f t="array" ref="E38">_xlfn.XLOOKUP(TRUE, EXACT(F38, Table1[orig]), Table1[(Y)])</f>
+        <v>U</v>
+      </c>
+      <c r="F38" t="str" cm="1">
+        <f t="array" ref="F38">_xlfn.XLOOKUP(TRUE, EXACT(G38, Table1[orig]), Table1[(Y)])</f>
+        <v>U</v>
+      </c>
+      <c r="G38" t="str" cm="1">
+        <f t="array" ref="G38">_xlfn.XLOOKUP(TRUE, EXACT(A38, Table1[orig]), Table1[(Y)])</f>
+        <v>U</v>
+      </c>
+      <c r="H38" t="str" cm="1">
+        <f t="array" ref="H38">_xlfn.XLOOKUP(TRUE, EXACT(I38, Table3[orig]), Table3[(Z)])</f>
+        <v>L</v>
+      </c>
+      <c r="I38" t="str" cm="1">
+        <f t="array" ref="I38">_xlfn.XLOOKUP(TRUE, EXACT(J38, Table3[orig]), Table3[(Z)])</f>
+        <v>D</v>
+      </c>
+      <c r="J38" t="str" cm="1">
+        <f t="array" ref="J38">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>R</v>
+      </c>
+      <c r="K38" t="str" cm="1">
+        <f t="array" ref="K38">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>U'</v>
+      </c>
+      <c r="L38" t="str" cm="1">
+        <f t="array" ref="L38">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>D'</v>
+      </c>
+      <c r="M38" t="str" cm="1">
+        <f t="array" ref="M38">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>U'</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A39" t="str">
+        <f>intermediate!E42</f>
+        <v>u</v>
+      </c>
+      <c r="B39" t="str" cm="1">
+        <f t="array" ref="B39">_xlfn.XLOOKUP(TRUE, EXACT(C39, Table4[orig]), Table4[(X)])</f>
+        <v>f</v>
+      </c>
+      <c r="C39" t="str" cm="1">
+        <f t="array" ref="C39">_xlfn.XLOOKUP(TRUE, EXACT(D39, Table4[orig]), Table4[(X)])</f>
+        <v>d</v>
+      </c>
+      <c r="D39" t="str" cm="1">
+        <f t="array" ref="D39">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>b</v>
+      </c>
+      <c r="E39" t="str" cm="1">
+        <f t="array" ref="E39">_xlfn.XLOOKUP(TRUE, EXACT(F39, Table1[orig]), Table1[(Y)])</f>
+        <v>u</v>
+      </c>
+      <c r="F39" t="str" cm="1">
+        <f t="array" ref="F39">_xlfn.XLOOKUP(TRUE, EXACT(G39, Table1[orig]), Table1[(Y)])</f>
+        <v>u</v>
+      </c>
+      <c r="G39" t="str" cm="1">
+        <f t="array" ref="G39">_xlfn.XLOOKUP(TRUE, EXACT(A39, Table1[orig]), Table1[(Y)])</f>
+        <v>u</v>
+      </c>
+      <c r="H39" t="str" cm="1">
+        <f t="array" ref="H39">_xlfn.XLOOKUP(TRUE, EXACT(I39, Table3[orig]), Table3[(Z)])</f>
+        <v>l</v>
+      </c>
+      <c r="I39" t="str" cm="1">
+        <f t="array" ref="I39">_xlfn.XLOOKUP(TRUE, EXACT(J39, Table3[orig]), Table3[(Z)])</f>
+        <v>d</v>
+      </c>
+      <c r="J39" t="str" cm="1">
+        <f t="array" ref="J39">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>r</v>
+      </c>
+      <c r="K39" t="str" cm="1">
+        <f t="array" ref="K39">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>u'</v>
+      </c>
+      <c r="L39" t="str" cm="1">
+        <f t="array" ref="L39">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>d'</v>
+      </c>
+      <c r="M39" t="str" cm="1">
+        <f t="array" ref="M39">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>u'</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A40" t="str">
+        <f>intermediate!E43</f>
+        <v>H</v>
+      </c>
+      <c r="B40" t="str" cm="1">
+        <f t="array" ref="B40">_xlfn.XLOOKUP(TRUE, EXACT(C40, Table4[orig]), Table4[(X)])</f>
+        <v>S</v>
+      </c>
+      <c r="C40" t="str" cm="1">
+        <f t="array" ref="C40">_xlfn.XLOOKUP(TRUE, EXACT(D40, Table4[orig]), Table4[(X)])</f>
+        <v>H'</v>
+      </c>
+      <c r="D40" t="str" cm="1">
+        <f t="array" ref="D40">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>S'</v>
+      </c>
+      <c r="E40" t="str" cm="1">
+        <f t="array" ref="E40">_xlfn.XLOOKUP(TRUE, EXACT(F40, Table1[orig]), Table1[(Y)])</f>
+        <v>H</v>
+      </c>
+      <c r="F40" t="str" cm="1">
+        <f t="array" ref="F40">_xlfn.XLOOKUP(TRUE, EXACT(G40, Table1[orig]), Table1[(Y)])</f>
+        <v>H</v>
+      </c>
+      <c r="G40" t="str" cm="1">
+        <f t="array" ref="G40">_xlfn.XLOOKUP(TRUE, EXACT(A40, Table1[orig]), Table1[(Y)])</f>
+        <v>H</v>
+      </c>
+      <c r="H40" t="str" cm="1">
+        <f t="array" ref="H40">_xlfn.XLOOKUP(TRUE, EXACT(I40, Table3[orig]), Table3[(Z)])</f>
+        <v>T'</v>
+      </c>
+      <c r="I40" t="str" cm="1">
+        <f t="array" ref="I40">_xlfn.XLOOKUP(TRUE, EXACT(J40, Table3[orig]), Table3[(Z)])</f>
+        <v>H'</v>
+      </c>
+      <c r="J40" t="str" cm="1">
+        <f t="array" ref="J40">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>T</v>
+      </c>
+      <c r="K40" t="str" cm="1">
+        <f t="array" ref="K40">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>H'</v>
+      </c>
+      <c r="L40" t="str" cm="1">
+        <f t="array" ref="L40">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>H</v>
+      </c>
+      <c r="M40" t="str" cm="1">
+        <f t="array" ref="M40">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>H'</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A41" t="str">
+        <f>intermediate!E44</f>
+        <v>d</v>
+      </c>
+      <c r="B41" t="str" cm="1">
+        <f t="array" ref="B41">_xlfn.XLOOKUP(TRUE, EXACT(C41, Table4[orig]), Table4[(X)])</f>
+        <v>b</v>
+      </c>
+      <c r="C41" t="str" cm="1">
+        <f t="array" ref="C41">_xlfn.XLOOKUP(TRUE, EXACT(D41, Table4[orig]), Table4[(X)])</f>
+        <v>u</v>
+      </c>
+      <c r="D41" t="str" cm="1">
+        <f t="array" ref="D41">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>f</v>
+      </c>
+      <c r="E41" t="str" cm="1">
+        <f t="array" ref="E41">_xlfn.XLOOKUP(TRUE, EXACT(F41, Table1[orig]), Table1[(Y)])</f>
+        <v>d</v>
+      </c>
+      <c r="F41" t="str" cm="1">
+        <f t="array" ref="F41">_xlfn.XLOOKUP(TRUE, EXACT(G41, Table1[orig]), Table1[(Y)])</f>
+        <v>d</v>
+      </c>
+      <c r="G41" t="str" cm="1">
+        <f t="array" ref="G41">_xlfn.XLOOKUP(TRUE, EXACT(A41, Table1[orig]), Table1[(Y)])</f>
+        <v>d</v>
+      </c>
+      <c r="H41" t="str" cm="1">
+        <f t="array" ref="H41">_xlfn.XLOOKUP(TRUE, EXACT(I41, Table3[orig]), Table3[(Z)])</f>
+        <v>r</v>
+      </c>
+      <c r="I41" t="str" cm="1">
+        <f t="array" ref="I41">_xlfn.XLOOKUP(TRUE, EXACT(J41, Table3[orig]), Table3[(Z)])</f>
+        <v>u</v>
+      </c>
+      <c r="J41" t="str" cm="1">
+        <f t="array" ref="J41">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>l</v>
+      </c>
+      <c r="K41" t="str" cm="1">
+        <f t="array" ref="K41">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>d'</v>
+      </c>
+      <c r="L41" t="str" cm="1">
+        <f t="array" ref="L41">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>u'</v>
+      </c>
+      <c r="M41" t="str" cm="1">
+        <f t="array" ref="M41">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>d'</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A42" t="str">
+        <f>intermediate!E45</f>
+        <v>D</v>
+      </c>
+      <c r="B42" t="str" cm="1">
+        <f t="array" ref="B42">_xlfn.XLOOKUP(TRUE, EXACT(C42, Table4[orig]), Table4[(X)])</f>
+        <v>B</v>
+      </c>
+      <c r="C42" t="str" cm="1">
+        <f t="array" ref="C42">_xlfn.XLOOKUP(TRUE, EXACT(D42, Table4[orig]), Table4[(X)])</f>
+        <v>U</v>
+      </c>
+      <c r="D42" t="str" cm="1">
+        <f t="array" ref="D42">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>F</v>
+      </c>
+      <c r="E42" t="str" cm="1">
+        <f t="array" ref="E42">_xlfn.XLOOKUP(TRUE, EXACT(F42, Table1[orig]), Table1[(Y)])</f>
+        <v>D</v>
+      </c>
+      <c r="F42" t="str" cm="1">
+        <f t="array" ref="F42">_xlfn.XLOOKUP(TRUE, EXACT(G42, Table1[orig]), Table1[(Y)])</f>
+        <v>D</v>
+      </c>
+      <c r="G42" t="str" cm="1">
+        <f t="array" ref="G42">_xlfn.XLOOKUP(TRUE, EXACT(A42, Table1[orig]), Table1[(Y)])</f>
+        <v>D</v>
+      </c>
+      <c r="H42" t="str" cm="1">
+        <f t="array" ref="H42">_xlfn.XLOOKUP(TRUE, EXACT(I42, Table3[orig]), Table3[(Z)])</f>
+        <v>R</v>
+      </c>
+      <c r="I42" t="str" cm="1">
+        <f t="array" ref="I42">_xlfn.XLOOKUP(TRUE, EXACT(J42, Table3[orig]), Table3[(Z)])</f>
+        <v>U</v>
+      </c>
+      <c r="J42" t="str" cm="1">
+        <f t="array" ref="J42">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>L</v>
+      </c>
+      <c r="K42" t="str" cm="1">
+        <f t="array" ref="K42">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>D'</v>
+      </c>
+      <c r="L42" t="str" cm="1">
+        <f t="array" ref="L42">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>U'</v>
+      </c>
+      <c r="M42" t="str" cm="1">
+        <f t="array" ref="M42">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>D'</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A43" s="3" t="str">
+        <f>intermediate!E46</f>
+        <v>Y</v>
+      </c>
+      <c r="B43" s="3" t="str" cm="1">
+        <f t="array" ref="B43">_xlfn.XLOOKUP(TRUE, EXACT(C43, Table4[orig]), Table4[(X)])</f>
+        <v>Z</v>
+      </c>
+      <c r="C43" s="3" t="str" cm="1">
+        <f t="array" ref="C43">_xlfn.XLOOKUP(TRUE, EXACT(D43, Table4[orig]), Table4[(X)])</f>
+        <v>Y'</v>
+      </c>
+      <c r="D43" s="3" t="str" cm="1">
+        <f t="array" ref="D43">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>Z'</v>
+      </c>
+      <c r="E43" s="3" t="str" cm="1">
+        <f t="array" ref="E43">_xlfn.XLOOKUP(TRUE, EXACT(F43, Table1[orig]), Table1[(Y)])</f>
+        <v>Y</v>
+      </c>
+      <c r="F43" s="3" t="str" cm="1">
+        <f t="array" ref="F43">_xlfn.XLOOKUP(TRUE, EXACT(G43, Table1[orig]), Table1[(Y)])</f>
+        <v>Y</v>
+      </c>
+      <c r="G43" s="3" t="str" cm="1">
+        <f t="array" ref="G43">_xlfn.XLOOKUP(TRUE, EXACT(A43, Table1[orig]), Table1[(Y)])</f>
+        <v>Y</v>
+      </c>
+      <c r="H43" s="3" t="str" cm="1">
+        <f t="array" ref="H43">_xlfn.XLOOKUP(TRUE, EXACT(I43, Table3[orig]), Table3[(Z)])</f>
+        <v>X'</v>
+      </c>
+      <c r="I43" s="3" t="str" cm="1">
+        <f t="array" ref="I43">_xlfn.XLOOKUP(TRUE, EXACT(J43, Table3[orig]), Table3[(Z)])</f>
+        <v>Y'</v>
+      </c>
+      <c r="J43" s="3" t="str" cm="1">
+        <f t="array" ref="J43">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>X</v>
+      </c>
+      <c r="K43" s="3" t="str" cm="1">
+        <f t="array" ref="K43">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>Y'</v>
+      </c>
+      <c r="L43" s="3" t="str" cm="1">
+        <f t="array" ref="L43">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>Y</v>
+      </c>
+      <c r="M43" s="3" t="str" cm="1">
+        <f t="array" ref="M43">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>Y'</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A44" t="str">
+        <f>intermediate!E47</f>
+        <v>U'</v>
+      </c>
+      <c r="B44" t="str" cm="1">
+        <f t="array" ref="B44">_xlfn.XLOOKUP(TRUE, EXACT(C44, Table4[orig]), Table4[(X)])</f>
+        <v>F'</v>
+      </c>
+      <c r="C44" t="str" cm="1">
+        <f t="array" ref="C44">_xlfn.XLOOKUP(TRUE, EXACT(D44, Table4[orig]), Table4[(X)])</f>
+        <v>D'</v>
+      </c>
+      <c r="D44" t="str" cm="1">
+        <f t="array" ref="D44">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>B'</v>
+      </c>
+      <c r="E44" t="str" cm="1">
+        <f t="array" ref="E44">_xlfn.XLOOKUP(TRUE, EXACT(F44, Table1[orig]), Table1[(Y)])</f>
+        <v>U'</v>
+      </c>
+      <c r="F44" t="str" cm="1">
+        <f t="array" ref="F44">_xlfn.XLOOKUP(TRUE, EXACT(G44, Table1[orig]), Table1[(Y)])</f>
+        <v>U'</v>
+      </c>
+      <c r="G44" t="str" cm="1">
+        <f t="array" ref="G44">_xlfn.XLOOKUP(TRUE, EXACT(A44, Table1[orig]), Table1[(Y)])</f>
+        <v>U'</v>
+      </c>
+      <c r="H44" t="str" cm="1">
+        <f t="array" ref="H44">_xlfn.XLOOKUP(TRUE, EXACT(I44, Table3[orig]), Table3[(Z)])</f>
+        <v>L'</v>
+      </c>
+      <c r="I44" t="str" cm="1">
+        <f t="array" ref="I44">_xlfn.XLOOKUP(TRUE, EXACT(J44, Table3[orig]), Table3[(Z)])</f>
+        <v>D'</v>
+      </c>
+      <c r="J44" t="str" cm="1">
+        <f t="array" ref="J44">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>R'</v>
+      </c>
+      <c r="K44" t="str" cm="1">
+        <f t="array" ref="K44">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>U</v>
+      </c>
+      <c r="L44" t="str" cm="1">
+        <f t="array" ref="L44">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>D</v>
+      </c>
+      <c r="M44" t="str" cm="1">
+        <f t="array" ref="M44">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>U</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A45" t="str">
+        <f>intermediate!E48</f>
+        <v>u'</v>
+      </c>
+      <c r="B45" t="str" cm="1">
+        <f t="array" ref="B45">_xlfn.XLOOKUP(TRUE, EXACT(C45, Table4[orig]), Table4[(X)])</f>
+        <v>f'</v>
+      </c>
+      <c r="C45" t="str" cm="1">
+        <f t="array" ref="C45">_xlfn.XLOOKUP(TRUE, EXACT(D45, Table4[orig]), Table4[(X)])</f>
+        <v>d'</v>
+      </c>
+      <c r="D45" t="str" cm="1">
+        <f t="array" ref="D45">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>b'</v>
+      </c>
+      <c r="E45" t="str" cm="1">
+        <f t="array" ref="E45">_xlfn.XLOOKUP(TRUE, EXACT(F45, Table1[orig]), Table1[(Y)])</f>
+        <v>u'</v>
+      </c>
+      <c r="F45" t="str" cm="1">
+        <f t="array" ref="F45">_xlfn.XLOOKUP(TRUE, EXACT(G45, Table1[orig]), Table1[(Y)])</f>
+        <v>u'</v>
+      </c>
+      <c r="G45" t="str" cm="1">
+        <f t="array" ref="G45">_xlfn.XLOOKUP(TRUE, EXACT(A45, Table1[orig]), Table1[(Y)])</f>
+        <v>u'</v>
+      </c>
+      <c r="H45" t="str" cm="1">
+        <f t="array" ref="H45">_xlfn.XLOOKUP(TRUE, EXACT(I45, Table3[orig]), Table3[(Z)])</f>
+        <v>l'</v>
+      </c>
+      <c r="I45" t="str" cm="1">
+        <f t="array" ref="I45">_xlfn.XLOOKUP(TRUE, EXACT(J45, Table3[orig]), Table3[(Z)])</f>
+        <v>d'</v>
+      </c>
+      <c r="J45" t="str" cm="1">
+        <f t="array" ref="J45">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>r'</v>
+      </c>
+      <c r="K45" t="str" cm="1">
+        <f t="array" ref="K45">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>u</v>
+      </c>
+      <c r="L45" t="str" cm="1">
+        <f t="array" ref="L45">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>d</v>
+      </c>
+      <c r="M45" t="str" cm="1">
+        <f t="array" ref="M45">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>u</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A46" t="str">
+        <f>intermediate!E49</f>
+        <v>H'</v>
+      </c>
+      <c r="B46" t="str" cm="1">
+        <f t="array" ref="B46">_xlfn.XLOOKUP(TRUE, EXACT(C46, Table4[orig]), Table4[(X)])</f>
+        <v>S'</v>
+      </c>
+      <c r="C46" t="str" cm="1">
+        <f t="array" ref="C46">_xlfn.XLOOKUP(TRUE, EXACT(D46, Table4[orig]), Table4[(X)])</f>
+        <v>H</v>
+      </c>
+      <c r="D46" t="str" cm="1">
+        <f t="array" ref="D46">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>S</v>
+      </c>
+      <c r="E46" t="str" cm="1">
+        <f t="array" ref="E46">_xlfn.XLOOKUP(TRUE, EXACT(F46, Table1[orig]), Table1[(Y)])</f>
+        <v>H'</v>
+      </c>
+      <c r="F46" t="str" cm="1">
+        <f t="array" ref="F46">_xlfn.XLOOKUP(TRUE, EXACT(G46, Table1[orig]), Table1[(Y)])</f>
+        <v>H'</v>
+      </c>
+      <c r="G46" t="str" cm="1">
+        <f t="array" ref="G46">_xlfn.XLOOKUP(TRUE, EXACT(A46, Table1[orig]), Table1[(Y)])</f>
+        <v>H'</v>
+      </c>
+      <c r="H46" t="str" cm="1">
+        <f t="array" ref="H46">_xlfn.XLOOKUP(TRUE, EXACT(I46, Table3[orig]), Table3[(Z)])</f>
+        <v>T</v>
+      </c>
+      <c r="I46" t="str" cm="1">
+        <f t="array" ref="I46">_xlfn.XLOOKUP(TRUE, EXACT(J46, Table3[orig]), Table3[(Z)])</f>
+        <v>H</v>
+      </c>
+      <c r="J46" t="str" cm="1">
+        <f t="array" ref="J46">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>T'</v>
+      </c>
+      <c r="K46" t="str" cm="1">
+        <f t="array" ref="K46">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>H</v>
+      </c>
+      <c r="L46" t="str" cm="1">
+        <f t="array" ref="L46">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>H'</v>
+      </c>
+      <c r="M46" t="str" cm="1">
+        <f t="array" ref="M46">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>H</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A47" t="str">
+        <f>intermediate!E50</f>
+        <v>d'</v>
+      </c>
+      <c r="B47" t="str" cm="1">
+        <f t="array" ref="B47">_xlfn.XLOOKUP(TRUE, EXACT(C47, Table4[orig]), Table4[(X)])</f>
+        <v>b'</v>
+      </c>
+      <c r="C47" t="str" cm="1">
+        <f t="array" ref="C47">_xlfn.XLOOKUP(TRUE, EXACT(D47, Table4[orig]), Table4[(X)])</f>
+        <v>u'</v>
+      </c>
+      <c r="D47" t="str" cm="1">
+        <f t="array" ref="D47">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>f'</v>
+      </c>
+      <c r="E47" t="str" cm="1">
+        <f t="array" ref="E47">_xlfn.XLOOKUP(TRUE, EXACT(F47, Table1[orig]), Table1[(Y)])</f>
+        <v>d'</v>
+      </c>
+      <c r="F47" t="str" cm="1">
+        <f t="array" ref="F47">_xlfn.XLOOKUP(TRUE, EXACT(G47, Table1[orig]), Table1[(Y)])</f>
+        <v>d'</v>
+      </c>
+      <c r="G47" t="str" cm="1">
+        <f t="array" ref="G47">_xlfn.XLOOKUP(TRUE, EXACT(A47, Table1[orig]), Table1[(Y)])</f>
+        <v>d'</v>
+      </c>
+      <c r="H47" t="str" cm="1">
+        <f t="array" ref="H47">_xlfn.XLOOKUP(TRUE, EXACT(I47, Table3[orig]), Table3[(Z)])</f>
+        <v>r'</v>
+      </c>
+      <c r="I47" t="str" cm="1">
+        <f t="array" ref="I47">_xlfn.XLOOKUP(TRUE, EXACT(J47, Table3[orig]), Table3[(Z)])</f>
+        <v>u'</v>
+      </c>
+      <c r="J47" t="str" cm="1">
+        <f t="array" ref="J47">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>l'</v>
+      </c>
+      <c r="K47" t="str" cm="1">
+        <f t="array" ref="K47">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>d</v>
+      </c>
+      <c r="L47" t="str" cm="1">
+        <f t="array" ref="L47">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>u</v>
+      </c>
+      <c r="M47" t="str" cm="1">
+        <f t="array" ref="M47">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>d</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A48" t="str">
+        <f>intermediate!E51</f>
+        <v>D'</v>
+      </c>
+      <c r="B48" t="str" cm="1">
+        <f t="array" ref="B48">_xlfn.XLOOKUP(TRUE, EXACT(C48, Table4[orig]), Table4[(X)])</f>
+        <v>B'</v>
+      </c>
+      <c r="C48" t="str" cm="1">
+        <f t="array" ref="C48">_xlfn.XLOOKUP(TRUE, EXACT(D48, Table4[orig]), Table4[(X)])</f>
+        <v>U'</v>
+      </c>
+      <c r="D48" t="str" cm="1">
+        <f t="array" ref="D48">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>F'</v>
+      </c>
+      <c r="E48" t="str" cm="1">
+        <f t="array" ref="E48">_xlfn.XLOOKUP(TRUE, EXACT(F48, Table1[orig]), Table1[(Y)])</f>
+        <v>D'</v>
+      </c>
+      <c r="F48" t="str" cm="1">
+        <f t="array" ref="F48">_xlfn.XLOOKUP(TRUE, EXACT(G48, Table1[orig]), Table1[(Y)])</f>
+        <v>D'</v>
+      </c>
+      <c r="G48" t="str" cm="1">
+        <f t="array" ref="G48">_xlfn.XLOOKUP(TRUE, EXACT(A48, Table1[orig]), Table1[(Y)])</f>
+        <v>D'</v>
+      </c>
+      <c r="H48" t="str" cm="1">
+        <f t="array" ref="H48">_xlfn.XLOOKUP(TRUE, EXACT(I48, Table3[orig]), Table3[(Z)])</f>
+        <v>R'</v>
+      </c>
+      <c r="I48" t="str" cm="1">
+        <f t="array" ref="I48">_xlfn.XLOOKUP(TRUE, EXACT(J48, Table3[orig]), Table3[(Z)])</f>
+        <v>U'</v>
+      </c>
+      <c r="J48" t="str" cm="1">
+        <f t="array" ref="J48">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>L'</v>
+      </c>
+      <c r="K48" t="str" cm="1">
+        <f t="array" ref="K48">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>D</v>
+      </c>
+      <c r="L48" t="str" cm="1">
+        <f t="array" ref="L48">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>U</v>
+      </c>
+      <c r="M48" t="str" cm="1">
+        <f t="array" ref="M48">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>D</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A49" s="3" t="str">
+        <f>intermediate!E52</f>
+        <v>Y'</v>
+      </c>
+      <c r="B49" s="3" t="str" cm="1">
+        <f t="array" ref="B49">_xlfn.XLOOKUP(TRUE, EXACT(C49, Table4[orig]), Table4[(X)])</f>
+        <v>Z'</v>
+      </c>
+      <c r="C49" s="3" t="str" cm="1">
+        <f t="array" ref="C49">_xlfn.XLOOKUP(TRUE, EXACT(D49, Table4[orig]), Table4[(X)])</f>
+        <v>Y</v>
+      </c>
+      <c r="D49" s="3" t="str" cm="1">
+        <f t="array" ref="D49">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>Z</v>
+      </c>
+      <c r="E49" s="3" t="str" cm="1">
+        <f t="array" ref="E49">_xlfn.XLOOKUP(TRUE, EXACT(F49, Table1[orig]), Table1[(Y)])</f>
+        <v>Y'</v>
+      </c>
+      <c r="F49" s="3" t="str" cm="1">
+        <f t="array" ref="F49">_xlfn.XLOOKUP(TRUE, EXACT(G49, Table1[orig]), Table1[(Y)])</f>
+        <v>Y'</v>
+      </c>
+      <c r="G49" s="3" t="str" cm="1">
+        <f t="array" ref="G49">_xlfn.XLOOKUP(TRUE, EXACT(A49, Table1[orig]), Table1[(Y)])</f>
+        <v>Y'</v>
+      </c>
+      <c r="H49" s="3" t="str" cm="1">
+        <f t="array" ref="H49">_xlfn.XLOOKUP(TRUE, EXACT(I49, Table3[orig]), Table3[(Z)])</f>
+        <v>X</v>
+      </c>
+      <c r="I49" s="3" t="str" cm="1">
+        <f t="array" ref="I49">_xlfn.XLOOKUP(TRUE, EXACT(J49, Table3[orig]), Table3[(Z)])</f>
+        <v>Y</v>
+      </c>
+      <c r="J49" s="3" t="str" cm="1">
+        <f t="array" ref="J49">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>X'</v>
+      </c>
+      <c r="K49" s="3" t="str" cm="1">
+        <f t="array" ref="K49">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>Y</v>
+      </c>
+      <c r="L49" s="3" t="str" cm="1">
+        <f t="array" ref="L49">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>Y'</v>
+      </c>
+      <c r="M49" s="3" t="str" cm="1">
+        <f t="array" ref="M49">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A50" t="str">
+        <f>intermediate!E53</f>
+        <v>U2</v>
+      </c>
+      <c r="B50" t="str" cm="1">
+        <f t="array" ref="B50">_xlfn.XLOOKUP(TRUE, EXACT(C50, Table4[orig]), Table4[(X)])</f>
+        <v>F2</v>
+      </c>
+      <c r="C50" t="str" cm="1">
+        <f t="array" ref="C50">_xlfn.XLOOKUP(TRUE, EXACT(D50, Table4[orig]), Table4[(X)])</f>
+        <v>D2</v>
+      </c>
+      <c r="D50" t="str" cm="1">
+        <f t="array" ref="D50">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>B2</v>
+      </c>
+      <c r="E50" t="str" cm="1">
+        <f t="array" ref="E50">_xlfn.XLOOKUP(TRUE, EXACT(F50, Table1[orig]), Table1[(Y)])</f>
+        <v>U2</v>
+      </c>
+      <c r="F50" t="str" cm="1">
+        <f t="array" ref="F50">_xlfn.XLOOKUP(TRUE, EXACT(G50, Table1[orig]), Table1[(Y)])</f>
+        <v>U2</v>
+      </c>
+      <c r="G50" t="str" cm="1">
+        <f t="array" ref="G50">_xlfn.XLOOKUP(TRUE, EXACT(A50, Table1[orig]), Table1[(Y)])</f>
+        <v>U2</v>
+      </c>
+      <c r="H50" t="str" cm="1">
+        <f t="array" ref="H50">_xlfn.XLOOKUP(TRUE, EXACT(I50, Table3[orig]), Table3[(Z)])</f>
+        <v>L2</v>
+      </c>
+      <c r="I50" t="str" cm="1">
+        <f t="array" ref="I50">_xlfn.XLOOKUP(TRUE, EXACT(J50, Table3[orig]), Table3[(Z)])</f>
+        <v>D2</v>
+      </c>
+      <c r="J50" t="str" cm="1">
+        <f t="array" ref="J50">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>R2</v>
+      </c>
+      <c r="K50" t="str" cm="1">
+        <f t="array" ref="K50">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>U2</v>
+      </c>
+      <c r="L50" t="str" cm="1">
+        <f t="array" ref="L50">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>D2</v>
+      </c>
+      <c r="M50" t="str" cm="1">
+        <f t="array" ref="M50">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>U2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A51" t="str">
+        <f>intermediate!E54</f>
+        <v>u2</v>
+      </c>
+      <c r="B51" t="str" cm="1">
+        <f t="array" ref="B51">_xlfn.XLOOKUP(TRUE, EXACT(C51, Table4[orig]), Table4[(X)])</f>
+        <v>f2</v>
+      </c>
+      <c r="C51" t="str" cm="1">
+        <f t="array" ref="C51">_xlfn.XLOOKUP(TRUE, EXACT(D51, Table4[orig]), Table4[(X)])</f>
+        <v>d2</v>
+      </c>
+      <c r="D51" t="str" cm="1">
+        <f t="array" ref="D51">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>b2</v>
+      </c>
+      <c r="E51" t="str" cm="1">
+        <f t="array" ref="E51">_xlfn.XLOOKUP(TRUE, EXACT(F51, Table1[orig]), Table1[(Y)])</f>
+        <v>u2</v>
+      </c>
+      <c r="F51" t="str" cm="1">
+        <f t="array" ref="F51">_xlfn.XLOOKUP(TRUE, EXACT(G51, Table1[orig]), Table1[(Y)])</f>
+        <v>u2</v>
+      </c>
+      <c r="G51" t="str" cm="1">
+        <f t="array" ref="G51">_xlfn.XLOOKUP(TRUE, EXACT(A51, Table1[orig]), Table1[(Y)])</f>
+        <v>u2</v>
+      </c>
+      <c r="H51" t="str" cm="1">
+        <f t="array" ref="H51">_xlfn.XLOOKUP(TRUE, EXACT(I51, Table3[orig]), Table3[(Z)])</f>
+        <v>l2</v>
+      </c>
+      <c r="I51" t="str" cm="1">
+        <f t="array" ref="I51">_xlfn.XLOOKUP(TRUE, EXACT(J51, Table3[orig]), Table3[(Z)])</f>
+        <v>d2</v>
+      </c>
+      <c r="J51" t="str" cm="1">
+        <f t="array" ref="J51">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>r2</v>
+      </c>
+      <c r="K51" t="str" cm="1">
+        <f t="array" ref="K51">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>u2</v>
+      </c>
+      <c r="L51" t="str" cm="1">
+        <f t="array" ref="L51">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>d2</v>
+      </c>
+      <c r="M51" t="str" cm="1">
+        <f t="array" ref="M51">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>u2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A52" t="str">
+        <f>intermediate!E55</f>
+        <v>H2</v>
+      </c>
+      <c r="B52" t="str" cm="1">
+        <f t="array" ref="B52">_xlfn.XLOOKUP(TRUE, EXACT(C52, Table4[orig]), Table4[(X)])</f>
+        <v>S2</v>
+      </c>
+      <c r="C52" t="str" cm="1">
+        <f t="array" ref="C52">_xlfn.XLOOKUP(TRUE, EXACT(D52, Table4[orig]), Table4[(X)])</f>
+        <v>H2</v>
+      </c>
+      <c r="D52" t="str" cm="1">
+        <f t="array" ref="D52">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>S2</v>
+      </c>
+      <c r="E52" t="str" cm="1">
+        <f t="array" ref="E52">_xlfn.XLOOKUP(TRUE, EXACT(F52, Table1[orig]), Table1[(Y)])</f>
+        <v>H2</v>
+      </c>
+      <c r="F52" t="str" cm="1">
+        <f t="array" ref="F52">_xlfn.XLOOKUP(TRUE, EXACT(G52, Table1[orig]), Table1[(Y)])</f>
+        <v>H2</v>
+      </c>
+      <c r="G52" t="str" cm="1">
+        <f t="array" ref="G52">_xlfn.XLOOKUP(TRUE, EXACT(A52, Table1[orig]), Table1[(Y)])</f>
+        <v>H2</v>
+      </c>
+      <c r="H52" t="str" cm="1">
+        <f t="array" ref="H52">_xlfn.XLOOKUP(TRUE, EXACT(I52, Table3[orig]), Table3[(Z)])</f>
+        <v>T2</v>
+      </c>
+      <c r="I52" t="str" cm="1">
+        <f t="array" ref="I52">_xlfn.XLOOKUP(TRUE, EXACT(J52, Table3[orig]), Table3[(Z)])</f>
+        <v>H2</v>
+      </c>
+      <c r="J52" t="str" cm="1">
+        <f t="array" ref="J52">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>T2</v>
+      </c>
+      <c r="K52" t="str" cm="1">
+        <f t="array" ref="K52">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>H2</v>
+      </c>
+      <c r="L52" t="str" cm="1">
+        <f t="array" ref="L52">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>H2</v>
+      </c>
+      <c r="M52" t="str" cm="1">
+        <f t="array" ref="M52">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>H2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A53" t="str">
+        <f>intermediate!E56</f>
+        <v>d2</v>
+      </c>
+      <c r="B53" t="str" cm="1">
+        <f t="array" ref="B53">_xlfn.XLOOKUP(TRUE, EXACT(C53, Table4[orig]), Table4[(X)])</f>
+        <v>b2</v>
+      </c>
+      <c r="C53" t="str" cm="1">
+        <f t="array" ref="C53">_xlfn.XLOOKUP(TRUE, EXACT(D53, Table4[orig]), Table4[(X)])</f>
+        <v>u2</v>
+      </c>
+      <c r="D53" t="str" cm="1">
+        <f t="array" ref="D53">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>f2</v>
+      </c>
+      <c r="E53" t="str" cm="1">
+        <f t="array" ref="E53">_xlfn.XLOOKUP(TRUE, EXACT(F53, Table1[orig]), Table1[(Y)])</f>
+        <v>d2</v>
+      </c>
+      <c r="F53" t="str" cm="1">
+        <f t="array" ref="F53">_xlfn.XLOOKUP(TRUE, EXACT(G53, Table1[orig]), Table1[(Y)])</f>
+        <v>d2</v>
+      </c>
+      <c r="G53" t="str" cm="1">
+        <f t="array" ref="G53">_xlfn.XLOOKUP(TRUE, EXACT(A53, Table1[orig]), Table1[(Y)])</f>
+        <v>d2</v>
+      </c>
+      <c r="H53" t="str" cm="1">
+        <f t="array" ref="H53">_xlfn.XLOOKUP(TRUE, EXACT(I53, Table3[orig]), Table3[(Z)])</f>
+        <v>r2</v>
+      </c>
+      <c r="I53" t="str" cm="1">
+        <f t="array" ref="I53">_xlfn.XLOOKUP(TRUE, EXACT(J53, Table3[orig]), Table3[(Z)])</f>
+        <v>u2</v>
+      </c>
+      <c r="J53" t="str" cm="1">
+        <f t="array" ref="J53">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>l2</v>
+      </c>
+      <c r="K53" t="str" cm="1">
+        <f t="array" ref="K53">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>d2</v>
+      </c>
+      <c r="L53" t="str" cm="1">
+        <f t="array" ref="L53">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>u2</v>
+      </c>
+      <c r="M53" t="str" cm="1">
+        <f t="array" ref="M53">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>d2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A54" t="str">
+        <f>intermediate!E57</f>
+        <v>D2</v>
+      </c>
+      <c r="B54" t="str" cm="1">
+        <f t="array" ref="B54">_xlfn.XLOOKUP(TRUE, EXACT(C54, Table4[orig]), Table4[(X)])</f>
+        <v>B2</v>
+      </c>
+      <c r="C54" t="str" cm="1">
+        <f t="array" ref="C54">_xlfn.XLOOKUP(TRUE, EXACT(D54, Table4[orig]), Table4[(X)])</f>
+        <v>U2</v>
+      </c>
+      <c r="D54" t="str" cm="1">
+        <f t="array" ref="D54">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>F2</v>
+      </c>
+      <c r="E54" t="str" cm="1">
+        <f t="array" ref="E54">_xlfn.XLOOKUP(TRUE, EXACT(F54, Table1[orig]), Table1[(Y)])</f>
+        <v>D2</v>
+      </c>
+      <c r="F54" t="str" cm="1">
+        <f t="array" ref="F54">_xlfn.XLOOKUP(TRUE, EXACT(G54, Table1[orig]), Table1[(Y)])</f>
+        <v>D2</v>
+      </c>
+      <c r="G54" t="str" cm="1">
+        <f t="array" ref="G54">_xlfn.XLOOKUP(TRUE, EXACT(A54, Table1[orig]), Table1[(Y)])</f>
+        <v>D2</v>
+      </c>
+      <c r="H54" t="str" cm="1">
+        <f t="array" ref="H54">_xlfn.XLOOKUP(TRUE, EXACT(I54, Table3[orig]), Table3[(Z)])</f>
+        <v>R2</v>
+      </c>
+      <c r="I54" t="str" cm="1">
+        <f t="array" ref="I54">_xlfn.XLOOKUP(TRUE, EXACT(J54, Table3[orig]), Table3[(Z)])</f>
+        <v>U2</v>
+      </c>
+      <c r="J54" t="str" cm="1">
+        <f t="array" ref="J54">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>L2</v>
+      </c>
+      <c r="K54" t="str" cm="1">
+        <f t="array" ref="K54">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>D2</v>
+      </c>
+      <c r="L54" t="str" cm="1">
+        <f t="array" ref="L54">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>U2</v>
+      </c>
+      <c r="M54" t="str" cm="1">
+        <f t="array" ref="M54">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>D2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A55" s="3" t="str">
+        <f>intermediate!E58</f>
+        <v>Y2</v>
+      </c>
+      <c r="B55" s="3" t="str" cm="1">
+        <f t="array" ref="B55">_xlfn.XLOOKUP(TRUE, EXACT(C55, Table4[orig]), Table4[(X)])</f>
+        <v>Z2</v>
+      </c>
+      <c r="C55" s="3" t="str" cm="1">
+        <f t="array" ref="C55">_xlfn.XLOOKUP(TRUE, EXACT(D55, Table4[orig]), Table4[(X)])</f>
+        <v>Y2</v>
+      </c>
+      <c r="D55" s="3" t="str" cm="1">
+        <f t="array" ref="D55">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table4[orig]), Table4[(X)])</f>
+        <v>Z2</v>
+      </c>
+      <c r="E55" s="3" t="str" cm="1">
+        <f t="array" ref="E55">_xlfn.XLOOKUP(TRUE, EXACT(F55, Table1[orig]), Table1[(Y)])</f>
+        <v>Y2</v>
+      </c>
+      <c r="F55" s="3" t="str" cm="1">
+        <f t="array" ref="F55">_xlfn.XLOOKUP(TRUE, EXACT(G55, Table1[orig]), Table1[(Y)])</f>
+        <v>Y2</v>
+      </c>
+      <c r="G55" s="3" t="str" cm="1">
+        <f t="array" ref="G55">_xlfn.XLOOKUP(TRUE, EXACT(A55, Table1[orig]), Table1[(Y)])</f>
+        <v>Y2</v>
+      </c>
+      <c r="H55" s="3" t="str" cm="1">
+        <f t="array" ref="H55">_xlfn.XLOOKUP(TRUE, EXACT(I55, Table3[orig]), Table3[(Z)])</f>
+        <v>X2</v>
+      </c>
+      <c r="I55" s="3" t="str" cm="1">
+        <f t="array" ref="I55">_xlfn.XLOOKUP(TRUE, EXACT(J55, Table3[orig]), Table3[(Z)])</f>
+        <v>Y2</v>
+      </c>
+      <c r="J55" s="3" t="str" cm="1">
+        <f t="array" ref="J55">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table3[orig]), Table3[(Z)])</f>
+        <v>X2</v>
+      </c>
+      <c r="K55" s="3" t="str" cm="1">
+        <f t="array" ref="K55">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table5[orig]), Table5[(T-reflection)])</f>
+        <v>Y2</v>
+      </c>
+      <c r="L55" s="3" t="str" cm="1">
+        <f t="array" ref="L55">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table6[orig]), Table6[(H-reflection)])</f>
+        <v>Y2</v>
+      </c>
+      <c r="M55" s="3" t="str" cm="1">
+        <f t="array" ref="M55">_xlfn.XLOOKUP(TRUE, EXACT(Table29[[#This Row],[orig]], Table7[orig]), Table7[(S-reflection)])</f>
+        <v>Y2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>